<commit_message>
Refine dual-strategy prediction UI and backend flow
</commit_message>
<xml_diff>
--- a/output/dayahead_price_prediction.xlsx
+++ b/output/dayahead_price_prediction.xlsx
@@ -495,13 +495,13 @@
         <v>292</v>
       </c>
       <c r="H2" t="n">
-        <v>267.6399264591799</v>
+        <v>270.9771237130446</v>
       </c>
       <c r="I2" t="n">
-        <v>33.43354797363281</v>
+        <v>-3.076587200164795</v>
       </c>
       <c r="J2" t="n">
-        <v>301.0734744328128</v>
+        <v>267.9005365128798</v>
       </c>
     </row>
     <row r="3">
@@ -531,13 +531,13 @@
         <v>289</v>
       </c>
       <c r="H3" t="n">
-        <v>264.4707665217906</v>
+        <v>267.8828540656346</v>
       </c>
       <c r="I3" t="n">
-        <v>31.93743515014648</v>
+        <v>-3.076587200164795</v>
       </c>
       <c r="J3" t="n">
-        <v>296.4082016719371</v>
+        <v>264.8062668654698</v>
       </c>
     </row>
     <row r="4">
@@ -567,13 +567,13 @@
         <v>288</v>
       </c>
       <c r="H4" t="n">
-        <v>263.8456680798847</v>
+        <v>271.3034772769633</v>
       </c>
       <c r="I4" t="n">
-        <v>24.4185962677002</v>
+        <v>-3.076587200164795</v>
       </c>
       <c r="J4" t="n">
-        <v>288.2642643475849</v>
+        <v>268.2268900767986</v>
       </c>
     </row>
     <row r="5">
@@ -603,13 +603,13 @@
         <v>285</v>
       </c>
       <c r="H5" t="n">
-        <v>262.9755368585136</v>
+        <v>270.1990539636352</v>
       </c>
       <c r="I5" t="n">
-        <v>24.03571319580078</v>
+        <v>-2.428779363632202</v>
       </c>
       <c r="J5" t="n">
-        <v>287.0112500543144</v>
+        <v>267.7702746000029</v>
       </c>
     </row>
     <row r="6">
@@ -639,13 +639,13 @@
         <v>295</v>
       </c>
       <c r="H6" t="n">
-        <v>260.0140265897415</v>
+        <v>260.6438318267952</v>
       </c>
       <c r="I6" t="n">
-        <v>24.03571319580078</v>
+        <v>-3.076587200164795</v>
       </c>
       <c r="J6" t="n">
-        <v>284.0497397855423</v>
+        <v>257.5672446266304</v>
       </c>
     </row>
     <row r="7">
@@ -675,13 +675,13 @@
         <v>289</v>
       </c>
       <c r="H7" t="n">
-        <v>258.5023235102862</v>
+        <v>262.4790491649094</v>
       </c>
       <c r="I7" t="n">
-        <v>19.82991218566895</v>
+        <v>-3.076587200164795</v>
       </c>
       <c r="J7" t="n">
-        <v>278.3322356959551</v>
+        <v>259.4024619647446</v>
       </c>
     </row>
     <row r="8">
@@ -711,13 +711,13 @@
         <v>280</v>
       </c>
       <c r="H8" t="n">
-        <v>259.6849697511161</v>
+        <v>261.8261233216266</v>
       </c>
       <c r="I8" t="n">
-        <v>21.51718139648438</v>
+        <v>-2.428779363632202</v>
       </c>
       <c r="J8" t="n">
-        <v>281.2021511476005</v>
+        <v>259.3973439579944</v>
       </c>
     </row>
     <row r="9">
@@ -747,13 +747,13 @@
         <v>289</v>
       </c>
       <c r="H9" t="n">
-        <v>263.7342924972236</v>
+        <v>271.1608350936759</v>
       </c>
       <c r="I9" t="n">
-        <v>21.51718139648438</v>
+        <v>-3.076587200164795</v>
       </c>
       <c r="J9" t="n">
-        <v>285.251473893708</v>
+        <v>268.0842478935111</v>
       </c>
     </row>
     <row r="10">
@@ -783,13 +783,13 @@
         <v>290</v>
       </c>
       <c r="H10" t="n">
-        <v>264.1329358475623</v>
+        <v>275.3140482845361</v>
       </c>
       <c r="I10" t="n">
-        <v>21.18766784667969</v>
+        <v>-3.076587200164795</v>
       </c>
       <c r="J10" t="n">
-        <v>285.320603694242</v>
+        <v>272.2374610843713</v>
       </c>
     </row>
     <row r="11">
@@ -819,13 +819,13 @@
         <v>285</v>
       </c>
       <c r="H11" t="n">
-        <v>264.2307156364269</v>
+        <v>270.397382741494</v>
       </c>
       <c r="I11" t="n">
-        <v>21.18766784667969</v>
+        <v>-2.428779363632202</v>
       </c>
       <c r="J11" t="n">
-        <v>285.4183834831065</v>
+        <v>267.9686033778618</v>
       </c>
     </row>
     <row r="12">
@@ -855,13 +855,13 @@
         <v>287</v>
       </c>
       <c r="H12" t="n">
-        <v>264.1726006803412</v>
+        <v>272.4093466226901</v>
       </c>
       <c r="I12" t="n">
-        <v>21.18766784667969</v>
+        <v>-3.076587200164795</v>
       </c>
       <c r="J12" t="n">
-        <v>285.3602685270209</v>
+        <v>269.3327594225253</v>
       </c>
     </row>
     <row r="13">
@@ -891,13 +891,13 @@
         <v>280</v>
       </c>
       <c r="H13" t="n">
-        <v>264.1814929085644</v>
+        <v>273.3378277828733</v>
       </c>
       <c r="I13" t="n">
-        <v>21.18766784667969</v>
+        <v>-2.428779363632202</v>
       </c>
       <c r="J13" t="n">
-        <v>285.3691607552441</v>
+        <v>270.9090484192411</v>
       </c>
     </row>
     <row r="14">
@@ -927,13 +927,13 @@
         <v>285</v>
       </c>
       <c r="H14" t="n">
-        <v>264.2673885025678</v>
+        <v>267.0500183047953</v>
       </c>
       <c r="I14" t="n">
-        <v>21.18766784667969</v>
+        <v>-2.428779363632202</v>
       </c>
       <c r="J14" t="n">
-        <v>285.4550563492475</v>
+        <v>264.6212389411631</v>
       </c>
     </row>
     <row r="15">
@@ -963,13 +963,13 @@
         <v>282</v>
       </c>
       <c r="H15" t="n">
-        <v>264.3009822075612</v>
+        <v>264.1945397459253</v>
       </c>
       <c r="I15" t="n">
-        <v>21.18766784667969</v>
+        <v>-2.428779363632202</v>
       </c>
       <c r="J15" t="n">
-        <v>285.4886500542408</v>
+        <v>261.7657603822931</v>
       </c>
     </row>
     <row r="16">
@@ -999,13 +999,13 @@
         <v>280</v>
       </c>
       <c r="H16" t="n">
-        <v>264.2362019969113</v>
+        <v>269.8561227224416</v>
       </c>
       <c r="I16" t="n">
-        <v>21.18766784667969</v>
+        <v>-2.428779363632202</v>
       </c>
       <c r="J16" t="n">
-        <v>285.423869843591</v>
+        <v>267.4273433588094</v>
       </c>
     </row>
     <row r="17">
@@ -1035,13 +1035,13 @@
         <v>285</v>
       </c>
       <c r="H17" t="n">
-        <v>264.3186819487491</v>
+        <v>262.6470387304171</v>
       </c>
       <c r="I17" t="n">
-        <v>21.18766784667969</v>
+        <v>-2.428779363632202</v>
       </c>
       <c r="J17" t="n">
-        <v>285.5063497954288</v>
+        <v>260.2182593667849</v>
       </c>
     </row>
     <row r="18">
@@ -1071,13 +1071,13 @@
         <v>280</v>
       </c>
       <c r="H18" t="n">
-        <v>264.3599716090519</v>
+        <v>263.2790945856014</v>
       </c>
       <c r="I18" t="n">
-        <v>21.18766784667969</v>
+        <v>-2.428779363632202</v>
       </c>
       <c r="J18" t="n">
-        <v>285.5476394557316</v>
+        <v>260.8503152219692</v>
       </c>
     </row>
     <row r="19">
@@ -1107,13 +1107,13 @@
         <v>280</v>
       </c>
       <c r="H19" t="n">
-        <v>264.4347294345513</v>
+        <v>266.8441232913817</v>
       </c>
       <c r="I19" t="n">
-        <v>21.18766784667969</v>
+        <v>-2.428779363632202</v>
       </c>
       <c r="J19" t="n">
-        <v>285.622397281231</v>
+        <v>264.4153439277495</v>
       </c>
     </row>
     <row r="20">
@@ -1143,13 +1143,13 @@
         <v>275</v>
       </c>
       <c r="H20" t="n">
-        <v>264.4007168080685</v>
+        <v>265.5852736845524</v>
       </c>
       <c r="I20" t="n">
-        <v>21.18766784667969</v>
+        <v>-2.428779363632202</v>
       </c>
       <c r="J20" t="n">
-        <v>285.5883846547482</v>
+        <v>263.1564943209202</v>
       </c>
     </row>
     <row r="21">
@@ -1179,13 +1179,13 @@
         <v>280</v>
       </c>
       <c r="H21" t="n">
-        <v>264.3866081638978</v>
+        <v>264.9255416950396</v>
       </c>
       <c r="I21" t="n">
-        <v>21.18766784667969</v>
+        <v>-2.428779363632202</v>
       </c>
       <c r="J21" t="n">
-        <v>285.5742760105775</v>
+        <v>262.4967623314074</v>
       </c>
     </row>
     <row r="22">
@@ -1215,13 +1215,13 @@
         <v>278</v>
       </c>
       <c r="H22" t="n">
-        <v>264.2672477714369</v>
+        <v>267.0620759064653</v>
       </c>
       <c r="I22" t="n">
-        <v>22.90105628967285</v>
+        <v>-2.428779363632202</v>
       </c>
       <c r="J22" t="n">
-        <v>287.1683040611098</v>
+        <v>264.6332965428331</v>
       </c>
     </row>
     <row r="23">
@@ -1251,13 +1251,13 @@
         <v>285</v>
       </c>
       <c r="H23" t="n">
-        <v>264.3111820359493</v>
+        <v>263.3103134059554</v>
       </c>
       <c r="I23" t="n">
-        <v>25.68872261047363</v>
+        <v>-2.428779363632202</v>
       </c>
       <c r="J23" t="n">
-        <v>289.9999046464229</v>
+        <v>260.8815340423232</v>
       </c>
     </row>
     <row r="24">
@@ -1287,13 +1287,13 @@
         <v>291</v>
       </c>
       <c r="H24" t="n">
-        <v>264.0666039113095</v>
+        <v>272.6096603857033</v>
       </c>
       <c r="I24" t="n">
-        <v>25.84806632995605</v>
+        <v>-3.076587200164795</v>
       </c>
       <c r="J24" t="n">
-        <v>289.9146702412656</v>
+        <v>269.5330731855385</v>
       </c>
     </row>
     <row r="25">
@@ -1323,13 +1323,13 @@
         <v>295</v>
       </c>
       <c r="H25" t="n">
-        <v>264.16186847644</v>
+        <v>285.2792925727875</v>
       </c>
       <c r="I25" t="n">
-        <v>26.05251693725586</v>
+        <v>-3.076587200164795</v>
       </c>
       <c r="J25" t="n">
-        <v>290.2143854136959</v>
+        <v>282.2027053726227</v>
       </c>
     </row>
     <row r="26">
@@ -1359,13 +1359,13 @@
         <v>292</v>
       </c>
       <c r="H26" t="n">
-        <v>264.0460017591008</v>
+        <v>272.6195352924882</v>
       </c>
       <c r="I26" t="n">
-        <v>28.20845985412598</v>
+        <v>-0.1309001743793488</v>
       </c>
       <c r="J26" t="n">
-        <v>292.2544616132268</v>
+        <v>272.4886351181088</v>
       </c>
     </row>
     <row r="27">
@@ -1395,13 +1395,13 @@
         <v>280</v>
       </c>
       <c r="H27" t="n">
-        <v>263.5657054640131</v>
+        <v>267.1701739253151</v>
       </c>
       <c r="I27" t="n">
-        <v>20.93247413635254</v>
+        <v>2.722239971160889</v>
       </c>
       <c r="J27" t="n">
-        <v>284.4981796003656</v>
+        <v>269.8924138964759</v>
       </c>
     </row>
     <row r="28">
@@ -1431,13 +1431,13 @@
         <v>279</v>
       </c>
       <c r="H28" t="n">
-        <v>259.4244565610407</v>
+        <v>262.0594182043163</v>
       </c>
       <c r="I28" t="n">
-        <v>21.5655517578125</v>
+        <v>-3.778454303741455</v>
       </c>
       <c r="J28" t="n">
-        <v>280.9900083188532</v>
+        <v>258.2809639005748</v>
       </c>
     </row>
     <row r="29">
@@ -1467,13 +1467,13 @@
         <v>275</v>
       </c>
       <c r="H29" t="n">
-        <v>248.2904504018086</v>
+        <v>252.7868926457715</v>
       </c>
       <c r="I29" t="n">
-        <v>29.0634822845459</v>
+        <v>-10.01123714447021</v>
       </c>
       <c r="J29" t="n">
-        <v>277.3539326863545</v>
+        <v>242.7756555013013</v>
       </c>
     </row>
     <row r="30">
@@ -1503,13 +1503,13 @@
         <v>270</v>
       </c>
       <c r="H30" t="n">
-        <v>249.7614796661608</v>
+        <v>250.8377136732146</v>
       </c>
       <c r="I30" t="n">
-        <v>21.04795074462891</v>
+        <v>-11.27502918243408</v>
       </c>
       <c r="J30" t="n">
-        <v>270.8094304107897</v>
+        <v>239.5626844907805</v>
       </c>
     </row>
     <row r="31">
@@ -1539,13 +1539,13 @@
         <v>264</v>
       </c>
       <c r="H31" t="n">
-        <v>240.1298876574091</v>
+        <v>254.8694311578868</v>
       </c>
       <c r="I31" t="n">
-        <v>17.61677742004397</v>
+        <v>-12.80007266998291</v>
       </c>
       <c r="J31" t="n">
-        <v>257.746665077453</v>
+        <v>242.0693584879039</v>
       </c>
     </row>
     <row r="32">
@@ -1575,13 +1575,13 @@
         <v>260</v>
       </c>
       <c r="H32" t="n">
-        <v>235.3193305843181</v>
+        <v>237.6064237832497</v>
       </c>
       <c r="I32" t="n">
-        <v>16.18205451965332</v>
+        <v>-13.46274948120117</v>
       </c>
       <c r="J32" t="n">
-        <v>251.5013851039714</v>
+        <v>224.1436743020486</v>
       </c>
     </row>
     <row r="33">
@@ -1611,13 +1611,13 @@
         <v>250</v>
       </c>
       <c r="H33" t="n">
-        <v>224.6332151027573</v>
+        <v>232.2227847094618</v>
       </c>
       <c r="I33" t="n">
-        <v>8.131274223327637</v>
+        <v>-13.46274948120117</v>
       </c>
       <c r="J33" t="n">
-        <v>232.7644893260849</v>
+        <v>218.7600352282606</v>
       </c>
     </row>
     <row r="34">
@@ -1647,13 +1647,13 @@
         <v>250</v>
       </c>
       <c r="H34" t="n">
-        <v>218.705691634483</v>
+        <v>251.3054032086596</v>
       </c>
       <c r="I34" t="n">
-        <v>4.66581916809082</v>
+        <v>-13.46274948120117</v>
       </c>
       <c r="J34" t="n">
-        <v>223.3715108025738</v>
+        <v>237.8426537274585</v>
       </c>
     </row>
     <row r="35">
@@ -1683,13 +1683,13 @@
         <v>245</v>
       </c>
       <c r="H35" t="n">
-        <v>220</v>
+        <v>195.3162106761534</v>
       </c>
       <c r="I35" t="n">
-        <v>-1.388814210891724</v>
+        <v>-26.22535514831543</v>
       </c>
       <c r="J35" t="n">
-        <v>218.6111857891082</v>
+        <v>169.090855527838</v>
       </c>
     </row>
     <row r="36">
@@ -1719,13 +1719,13 @@
         <v>235</v>
       </c>
       <c r="H36" t="n">
-        <v>150.747165327964</v>
+        <v>191.7149398695258</v>
       </c>
       <c r="I36" t="n">
-        <v>-6.328493595123291</v>
+        <v>-25.63429260253906</v>
       </c>
       <c r="J36" t="n">
-        <v>144.4186717328407</v>
+        <v>166.0806472669867</v>
       </c>
     </row>
     <row r="37">
@@ -1755,13 +1755,13 @@
         <v>210</v>
       </c>
       <c r="H37" t="n">
-        <v>130.2058887008976</v>
+        <v>197.5860820750164</v>
       </c>
       <c r="I37" t="n">
-        <v>-7.485358715057373</v>
+        <v>-25.63429260253906</v>
       </c>
       <c r="J37" t="n">
-        <v>122.7205299858402</v>
+        <v>171.9517894724774</v>
       </c>
     </row>
     <row r="38">
@@ -1791,13 +1791,13 @@
         <v>220</v>
       </c>
       <c r="H38" t="n">
-        <v>23.18160389670354</v>
+        <v>65.0202686423705</v>
       </c>
       <c r="I38" t="n">
-        <v>49.36655426025391</v>
+        <v>4.55800199508667</v>
       </c>
       <c r="J38" t="n">
-        <v>72.54815815695744</v>
+        <v>69.57827063745717</v>
       </c>
     </row>
     <row r="39">
@@ -1830,10 +1830,10 @@
         <v>139.8111972195845</v>
       </c>
       <c r="I39" t="n">
-        <v>-17.81954574584961</v>
+        <v>-3.112567901611328</v>
       </c>
       <c r="J39" t="n">
-        <v>121.9916514737349</v>
+        <v>136.6986293179732</v>
       </c>
     </row>
     <row r="40">
@@ -1866,10 +1866,10 @@
         <v>136.4747640811345</v>
       </c>
       <c r="I40" t="n">
-        <v>-13.31681346893311</v>
+        <v>-11.42272472381592</v>
       </c>
       <c r="J40" t="n">
-        <v>123.1579506122014</v>
+        <v>125.0520393573186</v>
       </c>
     </row>
     <row r="41">
@@ -1902,10 +1902,10 @@
         <v>133.2075525779215</v>
       </c>
       <c r="I41" t="n">
-        <v>-12.0822057723999</v>
+        <v>-3.112567901611328</v>
       </c>
       <c r="J41" t="n">
-        <v>121.1253468055216</v>
+        <v>130.0949846763101</v>
       </c>
     </row>
     <row r="42">
@@ -1935,13 +1935,13 @@
         <v>170</v>
       </c>
       <c r="H42" t="n">
-        <v>170.7514152460378</v>
+        <v>124.1960474812392</v>
       </c>
       <c r="I42" t="n">
-        <v>-32.55023193359375</v>
+        <v>-13.30914783477783</v>
       </c>
       <c r="J42" t="n">
-        <v>138.201183312444</v>
+        <v>110.8868996464614</v>
       </c>
     </row>
     <row r="43">
@@ -1971,13 +1971,13 @@
         <v>200</v>
       </c>
       <c r="H43" t="n">
-        <v>135.5985589276806</v>
+        <v>152.8726999912562</v>
       </c>
       <c r="I43" t="n">
-        <v>-32.55023193359375</v>
+        <v>-7.677032470703125</v>
       </c>
       <c r="J43" t="n">
-        <v>103.0483269940869</v>
+        <v>145.1956675205531</v>
       </c>
     </row>
     <row r="44">
@@ -2010,10 +2010,10 @@
         <v>55.90156675526624</v>
       </c>
       <c r="I44" t="n">
-        <v>49.59950637817382</v>
+        <v>34.28406906127929</v>
       </c>
       <c r="J44" t="n">
-        <v>105.5010731334401</v>
+        <v>90.18563581654553</v>
       </c>
     </row>
     <row r="45">
@@ -2043,13 +2043,13 @@
         <v>200</v>
       </c>
       <c r="H45" t="n">
-        <v>170.8480809790769</v>
+        <v>112.4814187673926</v>
       </c>
       <c r="I45" t="n">
-        <v>-32.55023193359375</v>
+        <v>18.62565040588379</v>
       </c>
       <c r="J45" t="n">
-        <v>138.2978490454831</v>
+        <v>131.1070691732764</v>
       </c>
     </row>
     <row r="46">
@@ -2082,10 +2082,10 @@
         <v>169.4551864602523</v>
       </c>
       <c r="I46" t="n">
-        <v>-32.55023193359375</v>
+        <v>16.53737640380859</v>
       </c>
       <c r="J46" t="n">
-        <v>136.9049545266586</v>
+        <v>185.9925628640609</v>
       </c>
     </row>
     <row r="47">
@@ -2115,13 +2115,13 @@
         <v>151</v>
       </c>
       <c r="H47" t="n">
-        <v>146.0307968727479</v>
+        <v>158.6685818240672</v>
       </c>
       <c r="I47" t="n">
-        <v>-32.55023193359375</v>
+        <v>15.84997653961182</v>
       </c>
       <c r="J47" t="n">
-        <v>113.4805649391542</v>
+        <v>174.518558363679</v>
       </c>
     </row>
     <row r="48">
@@ -2151,13 +2151,13 @@
         <v>200</v>
       </c>
       <c r="H48" t="n">
-        <v>176.327479295276</v>
+        <v>131.3655804996904</v>
       </c>
       <c r="I48" t="n">
-        <v>-34.99033355712891</v>
+        <v>-3.622000217437744</v>
       </c>
       <c r="J48" t="n">
-        <v>141.3371457381471</v>
+        <v>127.7435802822527</v>
       </c>
     </row>
     <row r="49">
@@ -2187,13 +2187,13 @@
         <v>200</v>
       </c>
       <c r="H49" t="n">
-        <v>54.59390290923398</v>
+        <v>56.74404221764922</v>
       </c>
       <c r="I49" t="n">
-        <v>37.1246109008789</v>
+        <v>44.52973556518555</v>
       </c>
       <c r="J49" t="n">
-        <v>91.71851381011288</v>
+        <v>101.2737777828348</v>
       </c>
     </row>
     <row r="50">
@@ -2223,13 +2223,13 @@
         <v>125</v>
       </c>
       <c r="H50" t="n">
-        <v>47.12385162306587</v>
+        <v>83.48077058176116</v>
       </c>
       <c r="I50" t="n">
-        <v>23.43623542785644</v>
+        <v>37.32822799682617</v>
       </c>
       <c r="J50" t="n">
-        <v>70.56008705092231</v>
+        <v>120.8089985785873</v>
       </c>
     </row>
     <row r="51">
@@ -2259,13 +2259,13 @@
         <v>0</v>
       </c>
       <c r="H51" t="n">
-        <v>47.63653964177303</v>
+        <v>77.19139563360383</v>
       </c>
       <c r="I51" t="n">
-        <v>25.42338943481445</v>
+        <v>33.11847686767578</v>
       </c>
       <c r="J51" t="n">
-        <v>73.05992907658748</v>
+        <v>110.3098725012796</v>
       </c>
     </row>
     <row r="52">
@@ -2295,13 +2295,13 @@
         <v>20</v>
       </c>
       <c r="H52" t="n">
-        <v>47.89117372358707</v>
+        <v>9.862601406240877</v>
       </c>
       <c r="I52" t="n">
-        <v>25.42338943481445</v>
+        <v>97.60361480712891</v>
       </c>
       <c r="J52" t="n">
-        <v>73.31456315840151</v>
+        <v>107.4662162133698</v>
       </c>
     </row>
     <row r="53">
@@ -2331,13 +2331,13 @@
         <v>0</v>
       </c>
       <c r="H53" t="n">
-        <v>47.96539736658031</v>
+        <v>13.15465337185785</v>
       </c>
       <c r="I53" t="n">
-        <v>24.76249313354491</v>
+        <v>44.68568801879883</v>
       </c>
       <c r="J53" t="n">
-        <v>72.72789050012523</v>
+        <v>57.84034139065668</v>
       </c>
     </row>
     <row r="54">
@@ -2367,13 +2367,13 @@
         <v>0</v>
       </c>
       <c r="H54" t="n">
-        <v>48.07158345158114</v>
+        <v>2.050349969194352</v>
       </c>
       <c r="I54" t="n">
-        <v>18.13446044921876</v>
+        <v>49.35341644287109</v>
       </c>
       <c r="J54" t="n">
-        <v>66.2060439007999</v>
+        <v>51.40376641206544</v>
       </c>
     </row>
     <row r="55">
@@ -2403,13 +2403,13 @@
         <v>170</v>
       </c>
       <c r="H55" t="n">
-        <v>48.18132485649422</v>
+        <v>16.15982473750876</v>
       </c>
       <c r="I55" t="n">
-        <v>13.34700489044189</v>
+        <v>72.06394958496094</v>
       </c>
       <c r="J55" t="n">
-        <v>61.52832974693612</v>
+        <v>88.22377432246969</v>
       </c>
     </row>
     <row r="56">
@@ -2439,13 +2439,13 @@
         <v>0</v>
       </c>
       <c r="H56" t="n">
-        <v>48.22165852123275</v>
+        <v>16.54761350150754</v>
       </c>
       <c r="I56" t="n">
-        <v>15.10599040985107</v>
+        <v>68.00099945068359</v>
       </c>
       <c r="J56" t="n">
-        <v>63.32764893108383</v>
+        <v>84.54861295219114</v>
       </c>
     </row>
     <row r="57">
@@ -2475,13 +2475,13 @@
         <v>125</v>
       </c>
       <c r="H57" t="n">
-        <v>48.23670332176044</v>
+        <v>15.24430438468193</v>
       </c>
       <c r="I57" t="n">
-        <v>13.1188325881958</v>
+        <v>70.22275543212891</v>
       </c>
       <c r="J57" t="n">
-        <v>61.35553590995624</v>
+        <v>85.46705981681083</v>
       </c>
     </row>
     <row r="58">
@@ -2511,13 +2511,13 @@
         <v>190</v>
       </c>
       <c r="H58" t="n">
-        <v>48.24311060140074</v>
+        <v>6.296304237898294</v>
       </c>
       <c r="I58" t="n">
-        <v>13.0532693862915</v>
+        <v>124.7493515014648</v>
       </c>
       <c r="J58" t="n">
-        <v>61.29637998769224</v>
+        <v>131.0456557393631</v>
       </c>
     </row>
     <row r="59">
@@ -2547,13 +2547,13 @@
         <v>215</v>
       </c>
       <c r="H59" t="n">
-        <v>48.24599298558167</v>
+        <v>4.253206729279307</v>
       </c>
       <c r="I59" t="n">
-        <v>8.884257316589355</v>
+        <v>69.73822021484375</v>
       </c>
       <c r="J59" t="n">
-        <v>57.13025030217103</v>
+        <v>73.99142694412306</v>
       </c>
     </row>
     <row r="60">
@@ -2583,13 +2583,13 @@
         <v>220</v>
       </c>
       <c r="H60" t="n">
-        <v>48.25805236651353</v>
+        <v>1.477898046014938</v>
       </c>
       <c r="I60" t="n">
-        <v>5.086898803710938</v>
+        <v>42.66005325317383</v>
       </c>
       <c r="J60" t="n">
-        <v>53.34495117022447</v>
+        <v>44.13795129918876</v>
       </c>
     </row>
     <row r="61">
@@ -2619,13 +2619,13 @@
         <v>220</v>
       </c>
       <c r="H61" t="n">
-        <v>48.26030335425847</v>
+        <v>2.991395176757578</v>
       </c>
       <c r="I61" t="n">
-        <v>-3.904783010482788</v>
+        <v>50.77659606933594</v>
       </c>
       <c r="J61" t="n">
-        <v>44.35552034377568</v>
+        <v>53.76799124609352</v>
       </c>
     </row>
     <row r="62">
@@ -2655,13 +2655,13 @@
         <v>229</v>
       </c>
       <c r="H62" t="n">
-        <v>48.25776325283894</v>
+        <v>1.286396647393492</v>
       </c>
       <c r="I62" t="n">
-        <v>6.30055570602417</v>
+        <v>13.17655849456787</v>
       </c>
       <c r="J62" t="n">
-        <v>54.55831895886311</v>
+        <v>14.46295514196136</v>
       </c>
     </row>
     <row r="63">
@@ -2691,13 +2691,13 @@
         <v>240</v>
       </c>
       <c r="H63" t="n">
-        <v>48.24853518760847</v>
+        <v>2.525826580078399</v>
       </c>
       <c r="I63" t="n">
-        <v>0.3952029645442963</v>
+        <v>13.17655849456787</v>
       </c>
       <c r="J63" t="n">
-        <v>48.64373815215277</v>
+        <v>15.70238507464627</v>
       </c>
     </row>
     <row r="64">
@@ -2727,13 +2727,13 @@
         <v>230</v>
       </c>
       <c r="H64" t="n">
-        <v>48.23911647095524</v>
+        <v>13.86339392899577</v>
       </c>
       <c r="I64" t="n">
-        <v>6.30055570602417</v>
+        <v>13.17655849456787</v>
       </c>
       <c r="J64" t="n">
-        <v>54.53967217697941</v>
+        <v>27.03995242356364</v>
       </c>
     </row>
     <row r="65">
@@ -2763,13 +2763,13 @@
         <v>250</v>
       </c>
       <c r="H65" t="n">
-        <v>48.22208147573301</v>
+        <v>16.89146254101057</v>
       </c>
       <c r="I65" t="n">
-        <v>0.3952029645442963</v>
+        <v>13.17655849456787</v>
       </c>
       <c r="J65" t="n">
-        <v>48.61728444027731</v>
+        <v>30.06802103557844</v>
       </c>
     </row>
     <row r="66">
@@ -2799,13 +2799,13 @@
         <v>245</v>
       </c>
       <c r="H66" t="n">
-        <v>48.20705974049991</v>
+        <v>2.613057667918365</v>
       </c>
       <c r="I66" t="n">
-        <v>0.3952029645442963</v>
+        <v>13.17655849456787</v>
       </c>
       <c r="J66" t="n">
-        <v>48.6022627050442</v>
+        <v>15.78961616248624</v>
       </c>
     </row>
     <row r="67">
@@ -2835,13 +2835,13 @@
         <v>265</v>
       </c>
       <c r="H67" t="n">
-        <v>47.88974454178815</v>
+        <v>9.836810347769731</v>
       </c>
       <c r="I67" t="n">
-        <v>15.37735462188721</v>
+        <v>13.17655849456787</v>
       </c>
       <c r="J67" t="n">
-        <v>63.26709916367535</v>
+        <v>23.0133688423376</v>
       </c>
     </row>
     <row r="68">
@@ -2871,13 +2871,13 @@
         <v>264</v>
       </c>
       <c r="H68" t="n">
-        <v>111.1196505572875</v>
+        <v>70.97261364809552</v>
       </c>
       <c r="I68" t="n">
-        <v>21.81804847717285</v>
+        <v>13.17655849456787</v>
       </c>
       <c r="J68" t="n">
-        <v>132.9376990344603</v>
+        <v>84.14917214266339</v>
       </c>
     </row>
     <row r="69">
@@ -2910,10 +2910,10 @@
         <v>166.1718364312146</v>
       </c>
       <c r="I69" t="n">
-        <v>0.07085421681404114</v>
+        <v>13.17655849456787</v>
       </c>
       <c r="J69" t="n">
-        <v>166.2426906480287</v>
+        <v>179.3483949257825</v>
       </c>
     </row>
     <row r="70">
@@ -2943,13 +2943,13 @@
         <v>295</v>
       </c>
       <c r="H70" t="n">
-        <v>26.73003772369167</v>
+        <v>202.4114561863755</v>
       </c>
       <c r="I70" t="n">
-        <v>21.81804847717285</v>
+        <v>13.17655849456787</v>
       </c>
       <c r="J70" t="n">
-        <v>48.54808620086452</v>
+        <v>215.5880146809434</v>
       </c>
     </row>
     <row r="71">
@@ -2979,13 +2979,13 @@
         <v>298</v>
       </c>
       <c r="H71" t="n">
-        <v>184.0450638803032</v>
+        <v>198.5029507999855</v>
       </c>
       <c r="I71" t="n">
-        <v>0.07085421681404114</v>
+        <v>13.17655849456787</v>
       </c>
       <c r="J71" t="n">
-        <v>184.1159180971173</v>
+        <v>211.6795092945534</v>
       </c>
     </row>
     <row r="72">
@@ -3015,13 +3015,13 @@
         <v>310</v>
       </c>
       <c r="H72" t="n">
-        <v>213.0960444488196</v>
+        <v>229.9912044684341</v>
       </c>
       <c r="I72" t="n">
-        <v>0.07085421681404114</v>
+        <v>13.17655849456787</v>
       </c>
       <c r="J72" t="n">
-        <v>213.1668986656337</v>
+        <v>243.167762963002</v>
       </c>
     </row>
     <row r="73">
@@ -3051,13 +3051,13 @@
         <v>310</v>
       </c>
       <c r="H73" t="n">
-        <v>239.3852217645793</v>
+        <v>276.6756074573791</v>
       </c>
       <c r="I73" t="n">
-        <v>0.07085421681404114</v>
+        <v>13.17655849456787</v>
       </c>
       <c r="J73" t="n">
-        <v>239.4560759813934</v>
+        <v>289.852165951947</v>
       </c>
     </row>
     <row r="74">
@@ -3087,13 +3087,13 @@
         <v>305</v>
       </c>
       <c r="H74" t="n">
-        <v>239.1450726185516</v>
+        <v>242.027387231861</v>
       </c>
       <c r="I74" t="n">
-        <v>-3.400023460388184</v>
+        <v>13.17655849456787</v>
       </c>
       <c r="J74" t="n">
-        <v>235.7450491581634</v>
+        <v>255.2039457264289</v>
       </c>
     </row>
     <row r="75">
@@ -3123,13 +3123,13 @@
         <v>305</v>
       </c>
       <c r="H75" t="n">
-        <v>248.2731623617452</v>
+        <v>258.3912237021769</v>
       </c>
       <c r="I75" t="n">
-        <v>-3.400023460388184</v>
+        <v>13.17655849456787</v>
       </c>
       <c r="J75" t="n">
-        <v>244.873138901357</v>
+        <v>271.5677821967448</v>
       </c>
     </row>
     <row r="76">
@@ -3159,13 +3159,13 @@
         <v>330</v>
       </c>
       <c r="H76" t="n">
-        <v>251.8283778868781</v>
+        <v>268.8675142042662</v>
       </c>
       <c r="I76" t="n">
-        <v>-3.300123691558838</v>
+        <v>13.17655849456787</v>
       </c>
       <c r="J76" t="n">
-        <v>248.5282541953193</v>
+        <v>282.044072698834</v>
       </c>
     </row>
     <row r="77">
@@ -3195,13 +3195,13 @@
         <v>339</v>
       </c>
       <c r="H77" t="n">
-        <v>264.4434456541305</v>
+        <v>273.7647282256407</v>
       </c>
       <c r="I77" t="n">
-        <v>-3.300123691558838</v>
+        <v>13.17655849456787</v>
       </c>
       <c r="J77" t="n">
-        <v>261.1433219625716</v>
+        <v>286.9412867202086</v>
       </c>
     </row>
     <row r="78">
@@ -3231,13 +3231,13 @@
         <v>328</v>
       </c>
       <c r="H78" t="n">
-        <v>264.1720749048455</v>
+        <v>272.3598865510795</v>
       </c>
       <c r="I78" t="n">
-        <v>-3.300123691558838</v>
+        <v>13.17655849456787</v>
       </c>
       <c r="J78" t="n">
-        <v>260.8719512132866</v>
+        <v>285.5364450456474</v>
       </c>
     </row>
     <row r="79">
@@ -3267,13 +3267,13 @@
         <v>325</v>
       </c>
       <c r="H79" t="n">
-        <v>264.0560532600432</v>
+        <v>265.3098230351048</v>
       </c>
       <c r="I79" t="n">
-        <v>-3.300123691558838</v>
+        <v>13.17655849456787</v>
       </c>
       <c r="J79" t="n">
-        <v>260.7559295684844</v>
+        <v>278.4863815296727</v>
       </c>
     </row>
     <row r="80">
@@ -3303,13 +3303,13 @@
         <v>325</v>
       </c>
       <c r="H80" t="n">
-        <v>265.5045212794324</v>
+        <v>271.2861954404619</v>
       </c>
       <c r="I80" t="n">
-        <v>-3.300123691558838</v>
+        <v>13.17655849456787</v>
       </c>
       <c r="J80" t="n">
-        <v>262.2043975878735</v>
+        <v>284.4627539350298</v>
       </c>
     </row>
     <row r="81">
@@ -3339,13 +3339,13 @@
         <v>318</v>
       </c>
       <c r="H81" t="n">
-        <v>264.7560004290006</v>
+        <v>270.4843253974767</v>
       </c>
       <c r="I81" t="n">
-        <v>-3.400023460388184</v>
+        <v>13.17655849456787</v>
       </c>
       <c r="J81" t="n">
-        <v>261.3559769686124</v>
+        <v>283.6608838920445</v>
       </c>
     </row>
     <row r="82">
@@ -3375,13 +3375,13 @@
         <v>313</v>
       </c>
       <c r="H82" t="n">
-        <v>264.5267664845981</v>
+        <v>269.8281208449547</v>
       </c>
       <c r="I82" t="n">
-        <v>15.10270595550537</v>
+        <v>7.415987968444824</v>
       </c>
       <c r="J82" t="n">
-        <v>279.6294724401035</v>
+        <v>277.2441088133995</v>
       </c>
     </row>
     <row r="83">
@@ -3411,13 +3411,13 @@
         <v>325</v>
       </c>
       <c r="H83" t="n">
-        <v>264.1374246827615</v>
+        <v>275.3007896207092</v>
       </c>
       <c r="I83" t="n">
-        <v>24.00565719604492</v>
+        <v>7.415987968444824</v>
       </c>
       <c r="J83" t="n">
-        <v>288.1430818788065</v>
+        <v>282.716777589154</v>
       </c>
     </row>
     <row r="84">
@@ -3447,13 +3447,13 @@
         <v>318</v>
       </c>
       <c r="H84" t="n">
-        <v>263.5318165323345</v>
+        <v>266.3351306546755</v>
       </c>
       <c r="I84" t="n">
-        <v>16.53445053100586</v>
+        <v>7.415987968444824</v>
       </c>
       <c r="J84" t="n">
-        <v>280.0662670633404</v>
+        <v>273.7511186231203</v>
       </c>
     </row>
     <row r="85">
@@ -3483,13 +3483,13 @@
         <v>318</v>
       </c>
       <c r="H85" t="n">
-        <v>262.2504450889737</v>
+        <v>263.8748987279326</v>
       </c>
       <c r="I85" t="n">
-        <v>18.98923873901367</v>
+        <v>7.415987968444824</v>
       </c>
       <c r="J85" t="n">
-        <v>281.2396838279873</v>
+        <v>271.2908866963774</v>
       </c>
     </row>
     <row r="86">
@@ -3519,13 +3519,13 @@
         <v>325</v>
       </c>
       <c r="H86" t="n">
-        <v>257.8748667315675</v>
+        <v>262.6333180197364</v>
       </c>
       <c r="I86" t="n">
-        <v>22.4882698059082</v>
+        <v>7.415987968444824</v>
       </c>
       <c r="J86" t="n">
-        <v>280.3631365374757</v>
+        <v>270.0493059881812</v>
       </c>
     </row>
     <row r="87">
@@ -3555,13 +3555,13 @@
         <v>300</v>
       </c>
       <c r="H87" t="n">
-        <v>247.9832908277266</v>
+        <v>276.3301368089377</v>
       </c>
       <c r="I87" t="n">
-        <v>18.40483093261722</v>
+        <v>7.415987968444824</v>
       </c>
       <c r="J87" t="n">
-        <v>266.3881217603438</v>
+        <v>283.7461247773825</v>
       </c>
     </row>
     <row r="88">
@@ -3591,13 +3591,13 @@
         <v>310</v>
       </c>
       <c r="H88" t="n">
-        <v>248.504095536432</v>
+        <v>257.8474278407156</v>
       </c>
       <c r="I88" t="n">
-        <v>18.66231918334964</v>
+        <v>7.415987968444824</v>
       </c>
       <c r="J88" t="n">
-        <v>267.1664147197816</v>
+        <v>265.2634158091604</v>
       </c>
     </row>
     <row r="89">
@@ -3627,13 +3627,13 @@
         <v>300</v>
       </c>
       <c r="H89" t="n">
-        <v>249.1512754809166</v>
+        <v>253.9053585257404</v>
       </c>
       <c r="I89" t="n">
-        <v>18.85830688476562</v>
+        <v>7.415987968444824</v>
       </c>
       <c r="J89" t="n">
-        <v>268.0095823656823</v>
+        <v>261.3213464941852</v>
       </c>
     </row>
     <row r="90">
@@ -3663,13 +3663,13 @@
         <v>298</v>
       </c>
       <c r="H90" t="n">
-        <v>236.5834995245432</v>
+        <v>237.1324135419671</v>
       </c>
       <c r="I90" t="n">
-        <v>19.82030105590817</v>
+        <v>7.415987968444824</v>
       </c>
       <c r="J90" t="n">
-        <v>256.4038005804514</v>
+        <v>244.5484015104119</v>
       </c>
     </row>
     <row r="91">
@@ -3699,13 +3699,13 @@
         <v>295</v>
       </c>
       <c r="H91" t="n">
-        <v>239.1838475905462</v>
+        <v>250.9996960943939</v>
       </c>
       <c r="I91" t="n">
-        <v>19.8203010559082</v>
+        <v>7.415987968444824</v>
       </c>
       <c r="J91" t="n">
-        <v>259.0041486464544</v>
+        <v>258.4156840628387</v>
       </c>
     </row>
     <row r="92">
@@ -3735,13 +3735,13 @@
         <v>292</v>
       </c>
       <c r="H92" t="n">
-        <v>235.683692499425</v>
+        <v>236.8127286496897</v>
       </c>
       <c r="I92" t="n">
-        <v>19.8203010559082</v>
+        <v>7.415987968444824</v>
       </c>
       <c r="J92" t="n">
-        <v>255.5039935553332</v>
+        <v>244.2287166181345</v>
       </c>
     </row>
     <row r="93">
@@ -3771,13 +3771,13 @@
         <v>290</v>
       </c>
       <c r="H93" t="n">
-        <v>223.5091780752699</v>
+        <v>229.6024077029018</v>
       </c>
       <c r="I93" t="n">
-        <v>19.8203010559082</v>
+        <v>7.415987968444824</v>
       </c>
       <c r="J93" t="n">
-        <v>243.3294791311781</v>
+        <v>237.0183956713466</v>
       </c>
     </row>
     <row r="94">
@@ -3807,13 +3807,13 @@
         <v>275</v>
       </c>
       <c r="H94" t="n">
-        <v>218.3533350987858</v>
+        <v>241.5170041167223</v>
       </c>
       <c r="I94" t="n">
-        <v>19.8203010559082</v>
+        <v>7.415987968444824</v>
       </c>
       <c r="J94" t="n">
-        <v>238.173636154694</v>
+        <v>248.9329920851671</v>
       </c>
     </row>
     <row r="95">
@@ -3843,13 +3843,13 @@
         <v>275</v>
       </c>
       <c r="H95" t="n">
-        <v>218.1009053984058</v>
+        <v>233.6456149299366</v>
       </c>
       <c r="I95" t="n">
-        <v>17.81948089599609</v>
+        <v>7.415987968444824</v>
       </c>
       <c r="J95" t="n">
-        <v>235.9203862944019</v>
+        <v>241.0616028983814</v>
       </c>
     </row>
     <row r="96">
@@ -3879,13 +3879,13 @@
         <v>270</v>
       </c>
       <c r="H96" t="n">
-        <v>219.7745048440841</v>
+        <v>221.5849831213032</v>
       </c>
       <c r="I96" t="n">
-        <v>17.1971321105957</v>
+        <v>7.415987968444824</v>
       </c>
       <c r="J96" t="n">
-        <v>236.9716369546798</v>
+        <v>229.000971089748</v>
       </c>
     </row>
     <row r="97">
@@ -3915,13 +3915,13 @@
         <v>270</v>
       </c>
       <c r="H97" t="n">
-        <v>217.645133044379</v>
+        <v>237.6219657425447</v>
       </c>
       <c r="I97" t="n">
-        <v>17.1971321105957</v>
+        <v>7.415987968444824</v>
       </c>
       <c r="J97" t="n">
-        <v>234.8422651549747</v>
+        <v>245.0379537109895</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Refine similarity features and persist training preferences
</commit_message>
<xml_diff>
--- a/output/dayahead_price_prediction.xlsx
+++ b/output/dayahead_price_prediction.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J97"/>
+  <dimension ref="A1:M97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,25 +444,40 @@
       </c>
       <c r="F1" t="inlineStr">
         <is>
+          <t>renewable_power</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
           <t>thermal_on_capacity</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>day_type</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
         <is>
           <t>lag_96</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>similar_price</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="K1" t="inlineStr">
+        <is>
+          <t>net_load_only_similar_price</t>
+        </is>
+      </c>
+      <c r="L1" t="inlineStr">
         <is>
           <t>residual_pred</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>predicted_price</t>
         </is>
@@ -489,19 +504,30 @@
         <v>24420.77</v>
       </c>
       <c r="F2" t="n">
-        <v>35095</v>
+        <v>7609.53</v>
       </c>
       <c r="G2" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H2" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I2" t="n">
         <v>292</v>
       </c>
-      <c r="H2" t="n">
-        <v>270.9771237130446</v>
-      </c>
-      <c r="I2" t="n">
-        <v>-3.076587200164795</v>
-      </c>
       <c r="J2" t="n">
-        <v>267.9005365128798</v>
+        <v>292</v>
+      </c>
+      <c r="K2" t="n">
+        <v>267.6399264591799</v>
+      </c>
+      <c r="L2" t="n">
+        <v>-2.090183258056641</v>
+      </c>
+      <c r="M2" t="n">
+        <v>289.9098167419434</v>
       </c>
     </row>
     <row r="3">
@@ -525,19 +551,30 @@
         <v>23719.18</v>
       </c>
       <c r="F3" t="n">
-        <v>35095</v>
+        <v>7467.12</v>
       </c>
       <c r="G3" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I3" t="n">
         <v>289</v>
       </c>
-      <c r="H3" t="n">
-        <v>267.8828540656346</v>
-      </c>
-      <c r="I3" t="n">
-        <v>-3.076587200164795</v>
-      </c>
       <c r="J3" t="n">
-        <v>264.8062668654698</v>
+        <v>289</v>
+      </c>
+      <c r="K3" t="n">
+        <v>264.4707665217906</v>
+      </c>
+      <c r="L3" t="n">
+        <v>-6.692414283752441</v>
+      </c>
+      <c r="M3" t="n">
+        <v>282.3075857162476</v>
       </c>
     </row>
     <row r="4">
@@ -561,19 +598,30 @@
         <v>23578.83</v>
       </c>
       <c r="F4" t="n">
-        <v>35095</v>
+        <v>7338.47</v>
       </c>
       <c r="G4" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I4" t="n">
         <v>288</v>
       </c>
-      <c r="H4" t="n">
-        <v>271.3034772769633</v>
-      </c>
-      <c r="I4" t="n">
-        <v>-3.076587200164795</v>
-      </c>
       <c r="J4" t="n">
-        <v>268.2268900767986</v>
+        <v>288</v>
+      </c>
+      <c r="K4" t="n">
+        <v>263.8456680798847</v>
+      </c>
+      <c r="L4" t="n">
+        <v>-4.75836706161499</v>
+      </c>
+      <c r="M4" t="n">
+        <v>283.241632938385</v>
       </c>
     </row>
     <row r="5">
@@ -597,19 +645,30 @@
         <v>23370</v>
       </c>
       <c r="F5" t="n">
-        <v>35095</v>
+        <v>7221.3</v>
       </c>
       <c r="G5" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I5" t="n">
         <v>285</v>
       </c>
-      <c r="H5" t="n">
-        <v>270.1990539636352</v>
-      </c>
-      <c r="I5" t="n">
-        <v>-2.428779363632202</v>
-      </c>
       <c r="J5" t="n">
-        <v>267.7702746000029</v>
+        <v>285</v>
+      </c>
+      <c r="K5" t="n">
+        <v>262.9755368585136</v>
+      </c>
+      <c r="L5" t="n">
+        <v>-0.2297959327697754</v>
+      </c>
+      <c r="M5" t="n">
+        <v>284.7702040672302</v>
       </c>
     </row>
     <row r="6">
@@ -633,19 +692,30 @@
         <v>23224.89</v>
       </c>
       <c r="F6" t="n">
-        <v>35095</v>
+        <v>7116.41</v>
       </c>
       <c r="G6" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H6" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I6" t="n">
         <v>295</v>
       </c>
-      <c r="H6" t="n">
-        <v>260.6438318267952</v>
-      </c>
-      <c r="I6" t="n">
-        <v>-3.076587200164795</v>
-      </c>
       <c r="J6" t="n">
-        <v>257.5672446266304</v>
+        <v>295</v>
+      </c>
+      <c r="K6" t="n">
+        <v>260.0140265897415</v>
+      </c>
+      <c r="L6" t="n">
+        <v>-11.96938419342041</v>
+      </c>
+      <c r="M6" t="n">
+        <v>283.0306158065796</v>
       </c>
     </row>
     <row r="7">
@@ -669,19 +739,30 @@
         <v>23012.53</v>
       </c>
       <c r="F7" t="n">
-        <v>35095</v>
+        <v>7020.77</v>
       </c>
       <c r="G7" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I7" t="n">
         <v>289</v>
       </c>
-      <c r="H7" t="n">
-        <v>262.4790491649094</v>
-      </c>
-      <c r="I7" t="n">
-        <v>-3.076587200164795</v>
-      </c>
       <c r="J7" t="n">
-        <v>259.4024619647446</v>
+        <v>289</v>
+      </c>
+      <c r="K7" t="n">
+        <v>258.5023235102862</v>
+      </c>
+      <c r="L7" t="n">
+        <v>-16.41978454589844</v>
+      </c>
+      <c r="M7" t="n">
+        <v>272.5802154541016</v>
       </c>
     </row>
     <row r="8">
@@ -705,19 +786,30 @@
         <v>23136.02</v>
       </c>
       <c r="F8" t="n">
-        <v>35095</v>
+        <v>6916.28</v>
       </c>
       <c r="G8" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I8" t="n">
         <v>280</v>
       </c>
-      <c r="H8" t="n">
-        <v>261.8261233216266</v>
-      </c>
-      <c r="I8" t="n">
-        <v>-2.428779363632202</v>
-      </c>
       <c r="J8" t="n">
-        <v>259.3973439579944</v>
+        <v>280</v>
+      </c>
+      <c r="K8" t="n">
+        <v>259.6849697511161</v>
+      </c>
+      <c r="L8" t="n">
+        <v>-3.58751916885376</v>
+      </c>
+      <c r="M8" t="n">
+        <v>276.4124808311462</v>
       </c>
     </row>
     <row r="9">
@@ -741,19 +833,30 @@
         <v>23605.39</v>
       </c>
       <c r="F9" t="n">
-        <v>35095</v>
+        <v>6811.91</v>
       </c>
       <c r="G9" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I9" t="n">
         <v>289</v>
       </c>
-      <c r="H9" t="n">
-        <v>271.1608350936759</v>
-      </c>
-      <c r="I9" t="n">
-        <v>-3.076587200164795</v>
-      </c>
       <c r="J9" t="n">
-        <v>268.0842478935111</v>
+        <v>289</v>
+      </c>
+      <c r="K9" t="n">
+        <v>263.7342924972236</v>
+      </c>
+      <c r="L9" t="n">
+        <v>-10.11219882965088</v>
+      </c>
+      <c r="M9" t="n">
+        <v>278.8878011703491</v>
       </c>
     </row>
     <row r="10">
@@ -777,19 +880,30 @@
         <v>23996.49</v>
       </c>
       <c r="F10" t="n">
-        <v>35095</v>
+        <v>6673.81</v>
       </c>
       <c r="G10" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I10" t="n">
         <v>290</v>
       </c>
-      <c r="H10" t="n">
-        <v>275.3140482845361</v>
-      </c>
-      <c r="I10" t="n">
-        <v>-3.076587200164795</v>
-      </c>
       <c r="J10" t="n">
-        <v>272.2374610843713</v>
+        <v>290</v>
+      </c>
+      <c r="K10" t="n">
+        <v>264.1329358475623</v>
+      </c>
+      <c r="L10" t="n">
+        <v>-8.420100212097168</v>
+      </c>
+      <c r="M10" t="n">
+        <v>281.5798997879028</v>
       </c>
     </row>
     <row r="11">
@@ -813,19 +927,30 @@
         <v>23901.14</v>
       </c>
       <c r="F11" t="n">
-        <v>35095</v>
+        <v>6540.46</v>
       </c>
       <c r="G11" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I11" t="n">
         <v>285</v>
       </c>
-      <c r="H11" t="n">
-        <v>270.397382741494</v>
-      </c>
-      <c r="I11" t="n">
-        <v>-2.428779363632202</v>
-      </c>
       <c r="J11" t="n">
-        <v>267.9686033778618</v>
+        <v>285</v>
+      </c>
+      <c r="K11" t="n">
+        <v>264.2307156364269</v>
+      </c>
+      <c r="L11" t="n">
+        <v>4.155219078063965</v>
+      </c>
+      <c r="M11" t="n">
+        <v>289.155219078064</v>
       </c>
     </row>
     <row r="12">
@@ -849,19 +974,30 @@
         <v>23956.05</v>
       </c>
       <c r="F12" t="n">
-        <v>35095</v>
+        <v>6391.05</v>
       </c>
       <c r="G12" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I12" t="n">
         <v>287</v>
       </c>
-      <c r="H12" t="n">
-        <v>272.4093466226901</v>
-      </c>
-      <c r="I12" t="n">
-        <v>-3.076587200164795</v>
-      </c>
       <c r="J12" t="n">
-        <v>269.3327594225253</v>
+        <v>287</v>
+      </c>
+      <c r="K12" t="n">
+        <v>264.1726006803412</v>
+      </c>
+      <c r="L12" t="n">
+        <v>-1.115578889846802</v>
+      </c>
+      <c r="M12" t="n">
+        <v>285.8844211101532</v>
       </c>
     </row>
     <row r="13">
@@ -885,19 +1021,30 @@
         <v>23947.32</v>
       </c>
       <c r="F13" t="n">
-        <v>35095</v>
+        <v>6229.68</v>
       </c>
       <c r="G13" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I13" t="n">
         <v>280</v>
       </c>
-      <c r="H13" t="n">
-        <v>273.3378277828733</v>
-      </c>
-      <c r="I13" t="n">
-        <v>-2.428779363632202</v>
-      </c>
       <c r="J13" t="n">
-        <v>270.9090484192411</v>
+        <v>280</v>
+      </c>
+      <c r="K13" t="n">
+        <v>264.1814929085644</v>
+      </c>
+      <c r="L13" t="n">
+        <v>4.155219078063965</v>
+      </c>
+      <c r="M13" t="n">
+        <v>284.155219078064</v>
       </c>
     </row>
     <row r="14">
@@ -921,19 +1068,30 @@
         <v>23868.97</v>
       </c>
       <c r="F14" t="n">
-        <v>35095</v>
+        <v>6100.13</v>
       </c>
       <c r="G14" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I14" t="n">
         <v>285</v>
       </c>
-      <c r="H14" t="n">
-        <v>267.0500183047953</v>
-      </c>
-      <c r="I14" t="n">
-        <v>-2.428779363632202</v>
-      </c>
       <c r="J14" t="n">
-        <v>264.6212389411631</v>
+        <v>285</v>
+      </c>
+      <c r="K14" t="n">
+        <v>264.2673885025678</v>
+      </c>
+      <c r="L14" t="n">
+        <v>3.293757915496826</v>
+      </c>
+      <c r="M14" t="n">
+        <v>288.2937579154968</v>
       </c>
     </row>
     <row r="15">
@@ -957,19 +1115,30 @@
         <v>23841.05</v>
       </c>
       <c r="F15" t="n">
-        <v>35095</v>
+        <v>5976.85</v>
       </c>
       <c r="G15" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I15" t="n">
         <v>282</v>
       </c>
-      <c r="H15" t="n">
-        <v>264.1945397459253</v>
-      </c>
-      <c r="I15" t="n">
-        <v>-2.428779363632202</v>
-      </c>
       <c r="J15" t="n">
-        <v>261.7657603822931</v>
+        <v>282</v>
+      </c>
+      <c r="K15" t="n">
+        <v>264.3009822075612</v>
+      </c>
+      <c r="L15" t="n">
+        <v>3.293757915496826</v>
+      </c>
+      <c r="M15" t="n">
+        <v>285.2937579154968</v>
       </c>
     </row>
     <row r="16">
@@ -993,19 +1162,30 @@
         <v>23896.21</v>
       </c>
       <c r="F16" t="n">
-        <v>35095</v>
+        <v>5864.99</v>
       </c>
       <c r="G16" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I16" t="n">
         <v>280</v>
       </c>
-      <c r="H16" t="n">
-        <v>269.8561227224416</v>
-      </c>
-      <c r="I16" t="n">
-        <v>-2.428779363632202</v>
-      </c>
       <c r="J16" t="n">
-        <v>267.4273433588094</v>
+        <v>280</v>
+      </c>
+      <c r="K16" t="n">
+        <v>264.2362019969113</v>
+      </c>
+      <c r="L16" t="n">
+        <v>4.155219078063965</v>
+      </c>
+      <c r="M16" t="n">
+        <v>284.155219078064</v>
       </c>
     </row>
     <row r="17">
@@ -1029,19 +1209,30 @@
         <v>23826.9</v>
       </c>
       <c r="F17" t="n">
-        <v>35095</v>
+        <v>5764.2</v>
       </c>
       <c r="G17" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I17" t="n">
         <v>285</v>
       </c>
-      <c r="H17" t="n">
-        <v>262.6470387304171</v>
-      </c>
-      <c r="I17" t="n">
-        <v>-2.428779363632202</v>
-      </c>
       <c r="J17" t="n">
-        <v>260.2182593667849</v>
+        <v>285</v>
+      </c>
+      <c r="K17" t="n">
+        <v>264.3186819487491</v>
+      </c>
+      <c r="L17" t="n">
+        <v>3.293757915496826</v>
+      </c>
+      <c r="M17" t="n">
+        <v>288.2937579154968</v>
       </c>
     </row>
     <row r="18">
@@ -1065,19 +1256,30 @@
         <v>23795.3</v>
       </c>
       <c r="F18" t="n">
-        <v>35095</v>
+        <v>5702.3</v>
       </c>
       <c r="G18" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I18" t="n">
         <v>280</v>
       </c>
-      <c r="H18" t="n">
-        <v>263.2790945856014</v>
-      </c>
-      <c r="I18" t="n">
-        <v>-2.428779363632202</v>
-      </c>
       <c r="J18" t="n">
-        <v>260.8503152219692</v>
+        <v>280</v>
+      </c>
+      <c r="K18" t="n">
+        <v>264.3599716090519</v>
+      </c>
+      <c r="L18" t="n">
+        <v>3.293757915496826</v>
+      </c>
+      <c r="M18" t="n">
+        <v>283.2937579154968</v>
       </c>
     </row>
     <row r="19">
@@ -1101,19 +1303,30 @@
         <v>23742.66</v>
       </c>
       <c r="F19" t="n">
-        <v>35095</v>
+        <v>5660.44</v>
       </c>
       <c r="G19" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I19" t="n">
         <v>280</v>
       </c>
-      <c r="H19" t="n">
-        <v>266.8441232913817</v>
-      </c>
-      <c r="I19" t="n">
-        <v>-2.428779363632202</v>
-      </c>
       <c r="J19" t="n">
-        <v>264.4153439277495</v>
+        <v>280</v>
+      </c>
+      <c r="K19" t="n">
+        <v>264.4347294345513</v>
+      </c>
+      <c r="L19" t="n">
+        <v>1.855008125305176</v>
+      </c>
+      <c r="M19" t="n">
+        <v>281.8550081253052</v>
       </c>
     </row>
     <row r="20">
@@ -1137,19 +1350,30 @@
         <v>23765.92</v>
       </c>
       <c r="F20" t="n">
-        <v>35095</v>
+        <v>5637.18</v>
       </c>
       <c r="G20" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I20" t="n">
         <v>275</v>
       </c>
-      <c r="H20" t="n">
-        <v>265.5852736845524</v>
-      </c>
-      <c r="I20" t="n">
-        <v>-2.428779363632202</v>
-      </c>
       <c r="J20" t="n">
-        <v>263.1564943209202</v>
+        <v>275</v>
+      </c>
+      <c r="K20" t="n">
+        <v>264.4007168080685</v>
+      </c>
+      <c r="L20" t="n">
+        <v>3.31649112701416</v>
+      </c>
+      <c r="M20" t="n">
+        <v>278.3164911270142</v>
       </c>
     </row>
     <row r="21">
@@ -1173,19 +1397,30 @@
         <v>23775.9</v>
       </c>
       <c r="F21" t="n">
-        <v>35095</v>
+        <v>5627.2</v>
       </c>
       <c r="G21" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I21" t="n">
         <v>280</v>
       </c>
-      <c r="H21" t="n">
-        <v>264.9255416950396</v>
-      </c>
-      <c r="I21" t="n">
-        <v>-2.428779363632202</v>
-      </c>
       <c r="J21" t="n">
-        <v>262.4967623314074</v>
+        <v>280</v>
+      </c>
+      <c r="K21" t="n">
+        <v>264.3866081638978</v>
+      </c>
+      <c r="L21" t="n">
+        <v>2.348443984985352</v>
+      </c>
+      <c r="M21" t="n">
+        <v>282.3484439849854</v>
       </c>
     </row>
     <row r="22">
@@ -1209,19 +1444,30 @@
         <v>23869.09</v>
       </c>
       <c r="F22" t="n">
-        <v>35095</v>
+        <v>5648.41</v>
       </c>
       <c r="G22" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I22" t="n">
         <v>278</v>
       </c>
-      <c r="H22" t="n">
-        <v>267.0620759064653</v>
-      </c>
-      <c r="I22" t="n">
-        <v>-2.428779363632202</v>
-      </c>
       <c r="J22" t="n">
-        <v>264.6332965428331</v>
+        <v>278</v>
+      </c>
+      <c r="K22" t="n">
+        <v>264.2672477714369</v>
+      </c>
+      <c r="L22" t="n">
+        <v>4.755241394042969</v>
+      </c>
+      <c r="M22" t="n">
+        <v>282.755241394043</v>
       </c>
     </row>
     <row r="23">
@@ -1245,19 +1491,30 @@
         <v>23832.85</v>
       </c>
       <c r="F23" t="n">
-        <v>35095</v>
+        <v>5701.35</v>
       </c>
       <c r="G23" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I23" t="n">
         <v>285</v>
       </c>
-      <c r="H23" t="n">
-        <v>263.3103134059554</v>
-      </c>
-      <c r="I23" t="n">
-        <v>-2.428779363632202</v>
-      </c>
       <c r="J23" t="n">
-        <v>260.8815340423232</v>
+        <v>285</v>
+      </c>
+      <c r="K23" t="n">
+        <v>264.3111820359493</v>
+      </c>
+      <c r="L23" t="n">
+        <v>4.234782695770264</v>
+      </c>
+      <c r="M23" t="n">
+        <v>289.2347826957703</v>
       </c>
     </row>
     <row r="24">
@@ -1281,19 +1538,30 @@
         <v>24069.2</v>
       </c>
       <c r="F24" t="n">
-        <v>35095</v>
+        <v>5805</v>
       </c>
       <c r="G24" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I24" t="n">
         <v>291</v>
       </c>
-      <c r="H24" t="n">
-        <v>272.6096603857033</v>
-      </c>
-      <c r="I24" t="n">
-        <v>-3.076587200164795</v>
-      </c>
       <c r="J24" t="n">
-        <v>269.5330731855385</v>
+        <v>291</v>
+      </c>
+      <c r="K24" t="n">
+        <v>264.0666039113095</v>
+      </c>
+      <c r="L24" t="n">
+        <v>-6.87318754196167</v>
+      </c>
+      <c r="M24" t="n">
+        <v>284.1268124580383</v>
       </c>
     </row>
     <row r="25">
@@ -1317,19 +1585,30 @@
         <v>24145.54</v>
       </c>
       <c r="F25" t="n">
-        <v>35095</v>
+        <v>6029.86</v>
       </c>
       <c r="G25" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I25" t="n">
         <v>295</v>
       </c>
-      <c r="H25" t="n">
-        <v>285.2792925727875</v>
-      </c>
-      <c r="I25" t="n">
-        <v>-3.076587200164795</v>
-      </c>
       <c r="J25" t="n">
-        <v>282.2027053726227</v>
+        <v>295</v>
+      </c>
+      <c r="K25" t="n">
+        <v>264.16186847644</v>
+      </c>
+      <c r="L25" t="n">
+        <v>-3.07116174697876</v>
+      </c>
+      <c r="M25" t="n">
+        <v>291.9288382530212</v>
       </c>
     </row>
     <row r="26">
@@ -1353,19 +1632,30 @@
         <v>24092.36</v>
       </c>
       <c r="F26" t="n">
-        <v>35095</v>
+        <v>6366.34</v>
       </c>
       <c r="G26" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I26" t="n">
         <v>292</v>
       </c>
-      <c r="H26" t="n">
-        <v>272.6195352924882</v>
-      </c>
-      <c r="I26" t="n">
-        <v>-0.1309001743793488</v>
-      </c>
       <c r="J26" t="n">
-        <v>272.4886351181088</v>
+        <v>292</v>
+      </c>
+      <c r="K26" t="n">
+        <v>264.0460017591008</v>
+      </c>
+      <c r="L26" t="n">
+        <v>33.51285934448242</v>
+      </c>
+      <c r="M26" t="n">
+        <v>325.5128593444824</v>
       </c>
     </row>
     <row r="27">
@@ -1389,19 +1679,30 @@
         <v>23673.16</v>
       </c>
       <c r="F27" t="n">
-        <v>35095</v>
+        <v>6841.24</v>
       </c>
       <c r="G27" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I27" t="n">
         <v>280</v>
       </c>
-      <c r="H27" t="n">
-        <v>267.1701739253151</v>
-      </c>
-      <c r="I27" t="n">
-        <v>2.722239971160889</v>
-      </c>
       <c r="J27" t="n">
-        <v>269.8924138964759</v>
+        <v>280</v>
+      </c>
+      <c r="K27" t="n">
+        <v>263.5657054640131</v>
+      </c>
+      <c r="L27" t="n">
+        <v>33.46404266357422</v>
+      </c>
+      <c r="M27" t="n">
+        <v>313.4640426635742</v>
       </c>
     </row>
     <row r="28">
@@ -1425,19 +1726,30 @@
         <v>23103.41</v>
       </c>
       <c r="F28" t="n">
-        <v>35095</v>
+        <v>7372.19</v>
       </c>
       <c r="G28" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I28" t="n">
         <v>279</v>
       </c>
-      <c r="H28" t="n">
-        <v>262.0594182043163</v>
-      </c>
-      <c r="I28" t="n">
-        <v>-3.778454303741455</v>
-      </c>
       <c r="J28" t="n">
-        <v>258.2809639005748</v>
+        <v>279</v>
+      </c>
+      <c r="K28" t="n">
+        <v>259.4244565610407</v>
+      </c>
+      <c r="L28" t="n">
+        <v>31.10340881347656</v>
+      </c>
+      <c r="M28" t="n">
+        <v>310.1034088134766</v>
       </c>
     </row>
     <row r="29">
@@ -1461,19 +1773,30 @@
         <v>22285.77</v>
       </c>
       <c r="F29" t="n">
-        <v>35095</v>
+        <v>7999.83</v>
       </c>
       <c r="G29" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I29" t="n">
         <v>275</v>
       </c>
-      <c r="H29" t="n">
-        <v>252.7868926457715</v>
-      </c>
-      <c r="I29" t="n">
-        <v>-10.01123714447021</v>
-      </c>
       <c r="J29" t="n">
-        <v>242.7756555013013</v>
+        <v>275</v>
+      </c>
+      <c r="K29" t="n">
+        <v>248.2904504018086</v>
+      </c>
+      <c r="L29" t="n">
+        <v>32.43955993652344</v>
+      </c>
+      <c r="M29" t="n">
+        <v>307.4395599365234</v>
       </c>
     </row>
     <row r="30">
@@ -1497,19 +1820,30 @@
         <v>21413.97</v>
       </c>
       <c r="F30" t="n">
-        <v>35095</v>
+        <v>8605.93</v>
       </c>
       <c r="G30" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I30" t="n">
         <v>270</v>
       </c>
-      <c r="H30" t="n">
-        <v>250.8377136732146</v>
-      </c>
-      <c r="I30" t="n">
-        <v>-11.27502918243408</v>
-      </c>
       <c r="J30" t="n">
-        <v>239.5626844907805</v>
+        <v>270</v>
+      </c>
+      <c r="K30" t="n">
+        <v>249.7614796661608</v>
+      </c>
+      <c r="L30" t="n">
+        <v>32.20755004882812</v>
+      </c>
+      <c r="M30" t="n">
+        <v>302.2075500488281</v>
       </c>
     </row>
     <row r="31">
@@ -1533,19 +1867,30 @@
         <v>20325.68</v>
       </c>
       <c r="F31" t="n">
-        <v>35095</v>
+        <v>9271.82</v>
       </c>
       <c r="G31" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I31" t="n">
         <v>264</v>
       </c>
-      <c r="H31" t="n">
-        <v>254.8694311578868</v>
-      </c>
-      <c r="I31" t="n">
-        <v>-12.80007266998291</v>
-      </c>
       <c r="J31" t="n">
-        <v>242.0693584879039</v>
+        <v>264</v>
+      </c>
+      <c r="K31" t="n">
+        <v>240.1298876574091</v>
+      </c>
+      <c r="L31" t="n">
+        <v>19.72584915161133</v>
+      </c>
+      <c r="M31" t="n">
+        <v>283.7258491516113</v>
       </c>
     </row>
     <row r="32">
@@ -1569,19 +1914,30 @@
         <v>19775.25</v>
       </c>
       <c r="F32" t="n">
-        <v>35095</v>
+        <v>9953.85</v>
       </c>
       <c r="G32" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I32" t="n">
         <v>260</v>
       </c>
-      <c r="H32" t="n">
-        <v>237.6064237832497</v>
-      </c>
-      <c r="I32" t="n">
-        <v>-13.46274948120117</v>
-      </c>
       <c r="J32" t="n">
-        <v>224.1436743020486</v>
+        <v>260</v>
+      </c>
+      <c r="K32" t="n">
+        <v>235.3193305843181</v>
+      </c>
+      <c r="L32" t="n">
+        <v>22.80068206787109</v>
+      </c>
+      <c r="M32" t="n">
+        <v>282.8006820678711</v>
       </c>
     </row>
     <row r="33">
@@ -1605,19 +1961,30 @@
         <v>19424.93</v>
       </c>
       <c r="F33" t="n">
-        <v>35095</v>
+        <v>10528.27</v>
       </c>
       <c r="G33" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I33" t="n">
         <v>250</v>
       </c>
-      <c r="H33" t="n">
-        <v>232.2227847094618</v>
-      </c>
-      <c r="I33" t="n">
-        <v>-13.46274948120117</v>
-      </c>
       <c r="J33" t="n">
-        <v>218.7600352282606</v>
+        <v>250</v>
+      </c>
+      <c r="K33" t="n">
+        <v>224.6332151027573</v>
+      </c>
+      <c r="L33" t="n">
+        <v>16.89102935791016</v>
+      </c>
+      <c r="M33" t="n">
+        <v>266.8910293579102</v>
       </c>
     </row>
     <row r="34">
@@ -1641,19 +2008,30 @@
         <v>19114.54</v>
       </c>
       <c r="F34" t="n">
-        <v>35095</v>
+        <v>11210.36</v>
       </c>
       <c r="G34" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I34" t="n">
         <v>250</v>
       </c>
-      <c r="H34" t="n">
-        <v>251.3054032086596</v>
-      </c>
-      <c r="I34" t="n">
-        <v>-13.46274948120117</v>
-      </c>
       <c r="J34" t="n">
-        <v>237.8426537274585</v>
+        <v>250</v>
+      </c>
+      <c r="K34" t="n">
+        <v>218.705691634483</v>
+      </c>
+      <c r="L34" t="n">
+        <v>12.81532287597656</v>
+      </c>
+      <c r="M34" t="n">
+        <v>262.8153228759766</v>
       </c>
     </row>
     <row r="35">
@@ -1677,19 +2055,30 @@
         <v>18636.27</v>
       </c>
       <c r="F35" t="n">
-        <v>35095</v>
+        <v>11900.33</v>
       </c>
       <c r="G35" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I35" t="n">
         <v>245</v>
       </c>
-      <c r="H35" t="n">
-        <v>195.3162106761534</v>
-      </c>
-      <c r="I35" t="n">
-        <v>-26.22535514831543</v>
-      </c>
       <c r="J35" t="n">
-        <v>169.090855527838</v>
+        <v>245</v>
+      </c>
+      <c r="K35" t="n">
+        <v>220</v>
+      </c>
+      <c r="L35" t="n">
+        <v>-0.01262378692626953</v>
+      </c>
+      <c r="M35" t="n">
+        <v>244.9873762130737</v>
       </c>
     </row>
     <row r="36">
@@ -1713,19 +2102,30 @@
         <v>18214.79</v>
       </c>
       <c r="F36" t="n">
-        <v>35095</v>
+        <v>12571.11</v>
       </c>
       <c r="G36" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I36" t="n">
         <v>235</v>
       </c>
-      <c r="H36" t="n">
-        <v>191.7149398695258</v>
-      </c>
-      <c r="I36" t="n">
-        <v>-25.63429260253906</v>
-      </c>
       <c r="J36" t="n">
-        <v>166.0806472669867</v>
+        <v>235</v>
+      </c>
+      <c r="K36" t="n">
+        <v>150.747165327964</v>
+      </c>
+      <c r="L36" t="n">
+        <v>-19.41651916503906</v>
+      </c>
+      <c r="M36" t="n">
+        <v>215.583480834961</v>
       </c>
     </row>
     <row r="37">
@@ -1749,19 +2149,30 @@
         <v>17803.05</v>
       </c>
       <c r="F37" t="n">
-        <v>35095</v>
+        <v>13175.45</v>
       </c>
       <c r="G37" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I37" t="n">
         <v>210</v>
       </c>
-      <c r="H37" t="n">
-        <v>197.5860820750164</v>
-      </c>
-      <c r="I37" t="n">
-        <v>-25.63429260253906</v>
-      </c>
       <c r="J37" t="n">
-        <v>171.9517894724774</v>
+        <v>210</v>
+      </c>
+      <c r="K37" t="n">
+        <v>130.2058887008976</v>
+      </c>
+      <c r="L37" t="n">
+        <v>-43.63359069824219</v>
+      </c>
+      <c r="M37" t="n">
+        <v>166.3664093017578</v>
       </c>
     </row>
     <row r="38">
@@ -1785,19 +2196,30 @@
         <v>17497.31</v>
       </c>
       <c r="F38" t="n">
-        <v>35095</v>
+        <v>13839.29</v>
       </c>
       <c r="G38" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I38" t="n">
         <v>220</v>
       </c>
-      <c r="H38" t="n">
-        <v>65.0202686423705</v>
-      </c>
-      <c r="I38" t="n">
-        <v>4.55800199508667</v>
-      </c>
       <c r="J38" t="n">
-        <v>69.57827063745717</v>
+        <v>220</v>
+      </c>
+      <c r="K38" t="n">
+        <v>23.18160389670354</v>
+      </c>
+      <c r="L38" t="n">
+        <v>-16.4579906463623</v>
+      </c>
+      <c r="M38" t="n">
+        <v>203.5420093536377</v>
       </c>
     </row>
     <row r="39">
@@ -1821,19 +2243,30 @@
         <v>17064</v>
       </c>
       <c r="F39" t="n">
-        <v>35095</v>
+        <v>14459.7</v>
       </c>
       <c r="G39" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I39" t="n">
         <v>0</v>
       </c>
-      <c r="H39" t="n">
+      <c r="J39" t="n">
+        <v>0</v>
+      </c>
+      <c r="K39" t="n">
         <v>139.8111972195845</v>
       </c>
-      <c r="I39" t="n">
-        <v>-3.112567901611328</v>
-      </c>
-      <c r="J39" t="n">
-        <v>136.6986293179732</v>
+      <c r="L39" t="n">
+        <v>48.88669967651367</v>
+      </c>
+      <c r="M39" t="n">
+        <v>48.88669967651367</v>
       </c>
     </row>
     <row r="40">
@@ -1857,19 +2290,30 @@
         <v>16725.53</v>
       </c>
       <c r="F40" t="n">
-        <v>35095</v>
+        <v>15042.97</v>
       </c>
       <c r="G40" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I40" t="n">
         <v>0</v>
       </c>
-      <c r="H40" t="n">
+      <c r="J40" t="n">
+        <v>0</v>
+      </c>
+      <c r="K40" t="n">
         <v>136.4747640811345</v>
       </c>
-      <c r="I40" t="n">
-        <v>-11.42272472381592</v>
-      </c>
-      <c r="J40" t="n">
-        <v>125.0520393573186</v>
+      <c r="L40" t="n">
+        <v>48.88669967651367</v>
+      </c>
+      <c r="M40" t="n">
+        <v>48.88669967651367</v>
       </c>
     </row>
     <row r="41">
@@ -1893,19 +2337,30 @@
         <v>17075.55</v>
       </c>
       <c r="F41" t="n">
-        <v>35095</v>
+        <v>15504.75</v>
       </c>
       <c r="G41" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I41" t="n">
         <v>0</v>
       </c>
-      <c r="H41" t="n">
+      <c r="J41" t="n">
+        <v>0</v>
+      </c>
+      <c r="K41" t="n">
         <v>133.2075525779215</v>
       </c>
-      <c r="I41" t="n">
-        <v>-3.112567901611328</v>
-      </c>
-      <c r="J41" t="n">
-        <v>130.0949846763101</v>
+      <c r="L41" t="n">
+        <v>48.88669967651367</v>
+      </c>
+      <c r="M41" t="n">
+        <v>48.88669967651367</v>
       </c>
     </row>
     <row r="42">
@@ -1929,19 +2384,30 @@
         <v>16978.2</v>
       </c>
       <c r="F42" t="n">
-        <v>35095</v>
+        <v>15947.4</v>
       </c>
       <c r="G42" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I42" t="n">
         <v>170</v>
       </c>
-      <c r="H42" t="n">
-        <v>124.1960474812392</v>
-      </c>
-      <c r="I42" t="n">
-        <v>-13.30914783477783</v>
-      </c>
       <c r="J42" t="n">
-        <v>110.8868996464614</v>
+        <v>170</v>
+      </c>
+      <c r="K42" t="n">
+        <v>170.7514152460378</v>
+      </c>
+      <c r="L42" t="n">
+        <v>-1.010861277580261</v>
+      </c>
+      <c r="M42" t="n">
+        <v>168.9891387224197</v>
       </c>
     </row>
     <row r="43">
@@ -1965,19 +2431,30 @@
         <v>17262.72</v>
       </c>
       <c r="F43" t="n">
-        <v>35095</v>
+        <v>16351.58</v>
       </c>
       <c r="G43" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I43" t="n">
         <v>200</v>
       </c>
-      <c r="H43" t="n">
-        <v>152.8726999912562</v>
-      </c>
-      <c r="I43" t="n">
-        <v>-7.677032470703125</v>
-      </c>
       <c r="J43" t="n">
-        <v>145.1956675205531</v>
+        <v>200</v>
+      </c>
+      <c r="K43" t="n">
+        <v>135.5985589276806</v>
+      </c>
+      <c r="L43" t="n">
+        <v>-5.468714237213135</v>
+      </c>
+      <c r="M43" t="n">
+        <v>194.5312857627869</v>
       </c>
     </row>
     <row r="44">
@@ -2001,19 +2478,30 @@
         <v>17191.42</v>
       </c>
       <c r="F44" t="n">
-        <v>35095</v>
+        <v>16696.68</v>
       </c>
       <c r="G44" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I44" t="n">
         <v>151</v>
       </c>
-      <c r="H44" t="n">
+      <c r="J44" t="n">
+        <v>151</v>
+      </c>
+      <c r="K44" t="n">
         <v>55.90156675526624</v>
       </c>
-      <c r="I44" t="n">
-        <v>34.28406906127929</v>
-      </c>
-      <c r="J44" t="n">
-        <v>90.18563581654553</v>
+      <c r="L44" t="n">
+        <v>-1.010861277580261</v>
+      </c>
+      <c r="M44" t="n">
+        <v>149.9891387224197</v>
       </c>
     </row>
     <row r="45">
@@ -2037,19 +2525,30 @@
         <v>16965.45</v>
       </c>
       <c r="F45" t="n">
-        <v>35095</v>
+        <v>16987.55</v>
       </c>
       <c r="G45" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I45" t="n">
         <v>200</v>
       </c>
-      <c r="H45" t="n">
-        <v>112.4814187673926</v>
-      </c>
-      <c r="I45" t="n">
-        <v>18.62565040588379</v>
-      </c>
       <c r="J45" t="n">
-        <v>131.1070691732764</v>
+        <v>200</v>
+      </c>
+      <c r="K45" t="n">
+        <v>170.8480809790769</v>
+      </c>
+      <c r="L45" t="n">
+        <v>-5.468714237213135</v>
+      </c>
+      <c r="M45" t="n">
+        <v>194.5312857627869</v>
       </c>
     </row>
     <row r="46">
@@ -2073,19 +2572,30 @@
         <v>16660</v>
       </c>
       <c r="F46" t="n">
-        <v>35095</v>
+        <v>17228.6</v>
       </c>
       <c r="G46" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H46" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I46" t="n">
         <v>151</v>
       </c>
-      <c r="H46" t="n">
+      <c r="J46" t="n">
+        <v>151</v>
+      </c>
+      <c r="K46" t="n">
         <v>169.4551864602523</v>
       </c>
-      <c r="I46" t="n">
-        <v>16.53737640380859</v>
-      </c>
-      <c r="J46" t="n">
-        <v>185.9925628640609</v>
+      <c r="L46" t="n">
+        <v>-1.010861277580261</v>
+      </c>
+      <c r="M46" t="n">
+        <v>149.9891387224197</v>
       </c>
     </row>
     <row r="47">
@@ -2109,19 +2619,30 @@
         <v>16391.88</v>
       </c>
       <c r="F47" t="n">
-        <v>35095</v>
+        <v>17477.22</v>
       </c>
       <c r="G47" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H47" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I47" t="n">
         <v>151</v>
       </c>
-      <c r="H47" t="n">
-        <v>158.6685818240672</v>
-      </c>
-      <c r="I47" t="n">
-        <v>15.84997653961182</v>
-      </c>
       <c r="J47" t="n">
-        <v>174.518558363679</v>
+        <v>151</v>
+      </c>
+      <c r="K47" t="n">
+        <v>146.0307968727479</v>
+      </c>
+      <c r="L47" t="n">
+        <v>-1.010861277580261</v>
+      </c>
+      <c r="M47" t="n">
+        <v>149.9891387224197</v>
       </c>
     </row>
     <row r="48">
@@ -2145,19 +2666,30 @@
         <v>16143.52</v>
       </c>
       <c r="F48" t="n">
-        <v>35095</v>
+        <v>17668.28</v>
       </c>
       <c r="G48" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H48" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I48" t="n">
         <v>200</v>
       </c>
-      <c r="H48" t="n">
-        <v>131.3655804996904</v>
-      </c>
-      <c r="I48" t="n">
-        <v>-3.622000217437744</v>
-      </c>
       <c r="J48" t="n">
-        <v>127.7435802822527</v>
+        <v>200</v>
+      </c>
+      <c r="K48" t="n">
+        <v>176.327479295276</v>
+      </c>
+      <c r="L48" t="n">
+        <v>-5.468714237213135</v>
+      </c>
+      <c r="M48" t="n">
+        <v>194.5312857627869</v>
       </c>
     </row>
     <row r="49">
@@ -2181,19 +2713,30 @@
         <v>15868.95</v>
       </c>
       <c r="F49" t="n">
-        <v>35095</v>
+        <v>17866.65</v>
       </c>
       <c r="G49" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H49" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I49" t="n">
         <v>200</v>
       </c>
-      <c r="H49" t="n">
-        <v>56.74404221764922</v>
-      </c>
-      <c r="I49" t="n">
-        <v>44.52973556518555</v>
-      </c>
       <c r="J49" t="n">
-        <v>101.2737777828348</v>
+        <v>200</v>
+      </c>
+      <c r="K49" t="n">
+        <v>54.59390290923398</v>
+      </c>
+      <c r="L49" t="n">
+        <v>-5.468714237213135</v>
+      </c>
+      <c r="M49" t="n">
+        <v>194.5312857627869</v>
       </c>
     </row>
     <row r="50">
@@ -2217,19 +2760,30 @@
         <v>15492.06</v>
       </c>
       <c r="F50" t="n">
-        <v>35095</v>
+        <v>18088.74</v>
       </c>
       <c r="G50" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H50" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I50" t="n">
         <v>125</v>
       </c>
-      <c r="H50" t="n">
-        <v>83.48077058176116</v>
-      </c>
-      <c r="I50" t="n">
-        <v>37.32822799682617</v>
-      </c>
       <c r="J50" t="n">
-        <v>120.8089985785873</v>
+        <v>125</v>
+      </c>
+      <c r="K50" t="n">
+        <v>47.12385162306587</v>
+      </c>
+      <c r="L50" t="n">
+        <v>36.3407440185547</v>
+      </c>
+      <c r="M50" t="n">
+        <v>161.3407440185547</v>
       </c>
     </row>
     <row r="51">
@@ -2253,19 +2807,30 @@
         <v>15392.73</v>
       </c>
       <c r="F51" t="n">
-        <v>35095</v>
+        <v>18279.37</v>
       </c>
       <c r="G51" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H51" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I51" t="n">
         <v>0</v>
       </c>
-      <c r="H51" t="n">
-        <v>77.19139563360383</v>
-      </c>
-      <c r="I51" t="n">
-        <v>33.11847686767578</v>
-      </c>
       <c r="J51" t="n">
-        <v>110.3098725012796</v>
+        <v>0</v>
+      </c>
+      <c r="K51" t="n">
+        <v>47.63653964177303</v>
+      </c>
+      <c r="L51" t="n">
+        <v>55.07820510864258</v>
+      </c>
+      <c r="M51" t="n">
+        <v>55.07820510864258</v>
       </c>
     </row>
     <row r="52">
@@ -2289,19 +2854,30 @@
         <v>15257.76</v>
       </c>
       <c r="F52" t="n">
-        <v>35095</v>
+        <v>18527.54</v>
       </c>
       <c r="G52" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H52" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I52" t="n">
         <v>20</v>
       </c>
-      <c r="H52" t="n">
-        <v>9.862601406240877</v>
-      </c>
-      <c r="I52" t="n">
-        <v>97.60361480712891</v>
-      </c>
       <c r="J52" t="n">
-        <v>107.4662162133698</v>
+        <v>20</v>
+      </c>
+      <c r="K52" t="n">
+        <v>47.89117372358707</v>
+      </c>
+      <c r="L52" t="n">
+        <v>55.57627868652344</v>
+      </c>
+      <c r="M52" t="n">
+        <v>75.57627868652344</v>
       </c>
     </row>
     <row r="53">
@@ -2325,19 +2901,30 @@
         <v>15183.25</v>
       </c>
       <c r="F53" t="n">
-        <v>35095</v>
+        <v>18695.35</v>
       </c>
       <c r="G53" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H53" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I53" t="n">
         <v>0</v>
       </c>
-      <c r="H53" t="n">
-        <v>13.15465337185785</v>
-      </c>
-      <c r="I53" t="n">
-        <v>44.68568801879883</v>
-      </c>
       <c r="J53" t="n">
-        <v>57.84034139065668</v>
+        <v>0</v>
+      </c>
+      <c r="K53" t="n">
+        <v>47.96539736658031</v>
+      </c>
+      <c r="L53" t="n">
+        <v>55.07820510864258</v>
+      </c>
+      <c r="M53" t="n">
+        <v>55.07820510864258</v>
       </c>
     </row>
     <row r="54">
@@ -2361,19 +2948,30 @@
         <v>15003.18</v>
       </c>
       <c r="F54" t="n">
-        <v>35095</v>
+        <v>18890.12</v>
       </c>
       <c r="G54" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H54" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I54" t="n">
         <v>0</v>
       </c>
-      <c r="H54" t="n">
-        <v>2.050349969194352</v>
-      </c>
-      <c r="I54" t="n">
-        <v>49.35341644287109</v>
-      </c>
       <c r="J54" t="n">
-        <v>51.40376641206544</v>
+        <v>0</v>
+      </c>
+      <c r="K54" t="n">
+        <v>48.07158345158114</v>
+      </c>
+      <c r="L54" t="n">
+        <v>55.07820510864258</v>
+      </c>
+      <c r="M54" t="n">
+        <v>55.07820510864258</v>
       </c>
     </row>
     <row r="55">
@@ -2397,19 +2995,30 @@
         <v>14552.72</v>
       </c>
       <c r="F55" t="n">
-        <v>35095</v>
+        <v>19051.08</v>
       </c>
       <c r="G55" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H55" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I55" t="n">
         <v>170</v>
       </c>
-      <c r="H55" t="n">
-        <v>16.15982473750876</v>
-      </c>
-      <c r="I55" t="n">
-        <v>72.06394958496094</v>
-      </c>
       <c r="J55" t="n">
-        <v>88.22377432246969</v>
+        <v>170</v>
+      </c>
+      <c r="K55" t="n">
+        <v>48.18132485649422</v>
+      </c>
+      <c r="L55" t="n">
+        <v>-15.23868942260742</v>
+      </c>
+      <c r="M55" t="n">
+        <v>154.7613105773926</v>
       </c>
     </row>
     <row r="56">
@@ -2433,19 +3042,30 @@
         <v>14164.67</v>
       </c>
       <c r="F56" t="n">
-        <v>35095</v>
+        <v>19188.43</v>
       </c>
       <c r="G56" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H56" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I56" t="n">
         <v>0</v>
       </c>
-      <c r="H56" t="n">
-        <v>16.54761350150754</v>
-      </c>
-      <c r="I56" t="n">
-        <v>68.00099945068359</v>
-      </c>
       <c r="J56" t="n">
-        <v>84.54861295219114</v>
+        <v>0</v>
+      </c>
+      <c r="K56" t="n">
+        <v>48.22165852123275</v>
+      </c>
+      <c r="L56" t="n">
+        <v>28.08449363708496</v>
+      </c>
+      <c r="M56" t="n">
+        <v>28.08449363708496</v>
       </c>
     </row>
     <row r="57">
@@ -2469,19 +3089,30 @@
         <v>13936.97</v>
       </c>
       <c r="F57" t="n">
-        <v>35095</v>
+        <v>19315.63</v>
       </c>
       <c r="G57" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H57" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I57" t="n">
         <v>125</v>
       </c>
-      <c r="H57" t="n">
-        <v>15.24430438468193</v>
-      </c>
-      <c r="I57" t="n">
-        <v>70.22275543212891</v>
-      </c>
       <c r="J57" t="n">
-        <v>85.46705981681083</v>
+        <v>125</v>
+      </c>
+      <c r="K57" t="n">
+        <v>48.23670332176044</v>
+      </c>
+      <c r="L57" t="n">
+        <v>-5.820196628570557</v>
+      </c>
+      <c r="M57" t="n">
+        <v>119.1798033714294</v>
       </c>
     </row>
     <row r="58">
@@ -2505,19 +3136,30 @@
         <v>13816.94</v>
       </c>
       <c r="F58" t="n">
-        <v>35095</v>
+        <v>19369.86</v>
       </c>
       <c r="G58" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H58" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I58" t="n">
         <v>190</v>
       </c>
-      <c r="H58" t="n">
-        <v>6.296304237898294</v>
-      </c>
-      <c r="I58" t="n">
-        <v>124.7493515014648</v>
-      </c>
       <c r="J58" t="n">
-        <v>131.0456557393631</v>
+        <v>190</v>
+      </c>
+      <c r="K58" t="n">
+        <v>48.24311060140074</v>
+      </c>
+      <c r="L58" t="n">
+        <v>-27.08765602111816</v>
+      </c>
+      <c r="M58" t="n">
+        <v>162.9123439788818</v>
       </c>
     </row>
     <row r="59">
@@ -2541,19 +3183,30 @@
         <v>13757.2</v>
       </c>
       <c r="F59" t="n">
-        <v>35095</v>
+        <v>19391.8</v>
       </c>
       <c r="G59" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H59" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I59" t="n">
         <v>215</v>
       </c>
-      <c r="H59" t="n">
-        <v>4.253206729279307</v>
-      </c>
-      <c r="I59" t="n">
-        <v>69.73822021484375</v>
-      </c>
       <c r="J59" t="n">
-        <v>73.99142694412306</v>
+        <v>215</v>
+      </c>
+      <c r="K59" t="n">
+        <v>48.24599298558167</v>
+      </c>
+      <c r="L59" t="n">
+        <v>-35.88713836669922</v>
+      </c>
+      <c r="M59" t="n">
+        <v>179.1128616333008</v>
       </c>
     </row>
     <row r="60">
@@ -2577,19 +3230,30 @@
         <v>13457.65</v>
       </c>
       <c r="F60" t="n">
-        <v>35095</v>
+        <v>19369.85</v>
       </c>
       <c r="G60" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H60" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I60" t="n">
         <v>220</v>
       </c>
-      <c r="H60" t="n">
-        <v>1.477898046014938</v>
-      </c>
-      <c r="I60" t="n">
-        <v>42.66005325317383</v>
-      </c>
       <c r="J60" t="n">
-        <v>44.13795129918876</v>
+        <v>220</v>
+      </c>
+      <c r="K60" t="n">
+        <v>48.25805236651353</v>
+      </c>
+      <c r="L60" t="n">
+        <v>-41.350830078125</v>
+      </c>
+      <c r="M60" t="n">
+        <v>178.649169921875</v>
       </c>
     </row>
     <row r="61">
@@ -2613,19 +3277,30 @@
         <v>13390.78</v>
       </c>
       <c r="F61" t="n">
-        <v>35095</v>
+        <v>19323.22</v>
       </c>
       <c r="G61" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H61" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I61" t="n">
         <v>220</v>
       </c>
-      <c r="H61" t="n">
-        <v>2.991395176757578</v>
-      </c>
-      <c r="I61" t="n">
-        <v>50.77659606933594</v>
-      </c>
       <c r="J61" t="n">
-        <v>53.76799124609352</v>
+        <v>220</v>
+      </c>
+      <c r="K61" t="n">
+        <v>48.26030335425847</v>
+      </c>
+      <c r="L61" t="n">
+        <v>-51.02811431884766</v>
+      </c>
+      <c r="M61" t="n">
+        <v>168.9718856811523</v>
       </c>
     </row>
     <row r="62">
@@ -2649,19 +3324,30 @@
         <v>13465.95</v>
       </c>
       <c r="F62" t="n">
-        <v>35095</v>
+        <v>19209.15</v>
       </c>
       <c r="G62" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H62" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I62" t="n">
         <v>229</v>
       </c>
-      <c r="H62" t="n">
-        <v>1.286396647393492</v>
-      </c>
-      <c r="I62" t="n">
-        <v>13.17655849456787</v>
-      </c>
       <c r="J62" t="n">
-        <v>14.46295514196136</v>
+        <v>229</v>
+      </c>
+      <c r="K62" t="n">
+        <v>48.25776325283894</v>
+      </c>
+      <c r="L62" t="n">
+        <v>7.761363506317139</v>
+      </c>
+      <c r="M62" t="n">
+        <v>236.7613635063171</v>
       </c>
     </row>
     <row r="63">
@@ -2685,19 +3371,30 @@
         <v>13701.14</v>
       </c>
       <c r="F63" t="n">
-        <v>35095</v>
+        <v>19070.06</v>
       </c>
       <c r="G63" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H63" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I63" t="n">
         <v>240</v>
       </c>
-      <c r="H63" t="n">
-        <v>2.525826580078399</v>
-      </c>
-      <c r="I63" t="n">
-        <v>13.17655849456787</v>
-      </c>
       <c r="J63" t="n">
-        <v>15.70238507464627</v>
+        <v>240</v>
+      </c>
+      <c r="K63" t="n">
+        <v>48.24853518760847</v>
+      </c>
+      <c r="L63" t="n">
+        <v>6.639773845672607</v>
+      </c>
+      <c r="M63" t="n">
+        <v>246.6397738456726</v>
       </c>
     </row>
     <row r="64">
@@ -2721,19 +3418,30 @@
         <v>13893.68</v>
       </c>
       <c r="F64" t="n">
-        <v>35095</v>
+        <v>18935.72</v>
       </c>
       <c r="G64" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H64" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I64" t="n">
         <v>230</v>
       </c>
-      <c r="H64" t="n">
-        <v>13.86339392899577</v>
-      </c>
-      <c r="I64" t="n">
-        <v>13.17655849456787</v>
-      </c>
       <c r="J64" t="n">
-        <v>27.03995242356364</v>
+        <v>230</v>
+      </c>
+      <c r="K64" t="n">
+        <v>48.23911647095524</v>
+      </c>
+      <c r="L64" t="n">
+        <v>7.761363506317139</v>
+      </c>
+      <c r="M64" t="n">
+        <v>237.7613635063171</v>
       </c>
     </row>
     <row r="65">
@@ -2757,19 +3465,30 @@
         <v>14159.11</v>
       </c>
       <c r="F65" t="n">
-        <v>35095</v>
+        <v>18804.09</v>
       </c>
       <c r="G65" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H65" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I65" t="n">
         <v>250</v>
       </c>
-      <c r="H65" t="n">
-        <v>16.89146254101057</v>
-      </c>
-      <c r="I65" t="n">
-        <v>13.17655849456787</v>
-      </c>
       <c r="J65" t="n">
-        <v>30.06802103557844</v>
+        <v>250</v>
+      </c>
+      <c r="K65" t="n">
+        <v>48.22208147573301</v>
+      </c>
+      <c r="L65" t="n">
+        <v>6.639773845672579</v>
+      </c>
+      <c r="M65" t="n">
+        <v>256.6397738456726</v>
       </c>
     </row>
     <row r="66">
@@ -2793,19 +3512,30 @@
         <v>14333.75</v>
       </c>
       <c r="F66" t="n">
-        <v>35095</v>
+        <v>18524.45</v>
       </c>
       <c r="G66" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H66" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I66" t="n">
         <v>245</v>
       </c>
-      <c r="H66" t="n">
-        <v>2.613057667918365</v>
-      </c>
-      <c r="I66" t="n">
-        <v>13.17655849456787</v>
-      </c>
       <c r="J66" t="n">
-        <v>15.78961616248624</v>
+        <v>245</v>
+      </c>
+      <c r="K66" t="n">
+        <v>48.20705974049991</v>
+      </c>
+      <c r="L66" t="n">
+        <v>6.639773845672607</v>
+      </c>
+      <c r="M66" t="n">
+        <v>251.6397738456726</v>
       </c>
     </row>
     <row r="67">
@@ -2829,19 +3559,30 @@
         <v>15258.95</v>
       </c>
       <c r="F67" t="n">
-        <v>35095</v>
+        <v>18184.55</v>
       </c>
       <c r="G67" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H67" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I67" t="n">
         <v>265</v>
       </c>
-      <c r="H67" t="n">
-        <v>9.836810347769731</v>
-      </c>
-      <c r="I67" t="n">
-        <v>13.17655849456787</v>
-      </c>
       <c r="J67" t="n">
-        <v>23.0133688423376</v>
+        <v>265</v>
+      </c>
+      <c r="K67" t="n">
+        <v>47.88974454178815</v>
+      </c>
+      <c r="L67" t="n">
+        <v>6.639773845672607</v>
+      </c>
+      <c r="M67" t="n">
+        <v>271.6397738456726</v>
       </c>
     </row>
     <row r="68">
@@ -2865,19 +3606,30 @@
         <v>15896.49</v>
       </c>
       <c r="F68" t="n">
-        <v>35095</v>
+        <v>17800.71</v>
       </c>
       <c r="G68" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H68" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I68" t="n">
         <v>264</v>
       </c>
-      <c r="H68" t="n">
-        <v>70.97261364809552</v>
-      </c>
-      <c r="I68" t="n">
-        <v>13.17655849456787</v>
-      </c>
       <c r="J68" t="n">
-        <v>84.14917214266339</v>
+        <v>264</v>
+      </c>
+      <c r="K68" t="n">
+        <v>111.1196505572875</v>
+      </c>
+      <c r="L68" t="n">
+        <v>6.639773845672607</v>
+      </c>
+      <c r="M68" t="n">
+        <v>270.6397738456726</v>
       </c>
     </row>
     <row r="69">
@@ -2901,19 +3653,30 @@
         <v>16666.24</v>
       </c>
       <c r="F69" t="n">
-        <v>35095</v>
+        <v>17375.56</v>
       </c>
       <c r="G69" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H69" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I69" t="n">
         <v>278</v>
       </c>
-      <c r="H69" t="n">
+      <c r="J69" t="n">
+        <v>278</v>
+      </c>
+      <c r="K69" t="n">
         <v>166.1718364312146</v>
       </c>
-      <c r="I69" t="n">
-        <v>13.17655849456787</v>
-      </c>
-      <c r="J69" t="n">
-        <v>179.3483949257825</v>
+      <c r="L69" t="n">
+        <v>1.320194721221924</v>
+      </c>
+      <c r="M69" t="n">
+        <v>279.3201947212219</v>
       </c>
     </row>
     <row r="70">
@@ -2937,19 +3700,30 @@
         <v>17444.52</v>
       </c>
       <c r="F70" t="n">
-        <v>35095</v>
+        <v>16816.88</v>
       </c>
       <c r="G70" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H70" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I70" t="n">
         <v>295</v>
       </c>
-      <c r="H70" t="n">
-        <v>202.4114561863755</v>
-      </c>
-      <c r="I70" t="n">
-        <v>13.17655849456787</v>
-      </c>
       <c r="J70" t="n">
-        <v>215.5880146809434</v>
+        <v>295</v>
+      </c>
+      <c r="K70" t="n">
+        <v>26.73003772369167</v>
+      </c>
+      <c r="L70" t="n">
+        <v>-3.630966901779175</v>
+      </c>
+      <c r="M70" t="n">
+        <v>291.3690330982208</v>
       </c>
     </row>
     <row r="71">
@@ -2973,19 +3747,30 @@
         <v>18387.13</v>
       </c>
       <c r="F71" t="n">
-        <v>35095</v>
+        <v>16198.77</v>
       </c>
       <c r="G71" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H71" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I71" t="n">
         <v>298</v>
       </c>
-      <c r="H71" t="n">
-        <v>198.5029507999855</v>
-      </c>
-      <c r="I71" t="n">
-        <v>13.17655849456787</v>
-      </c>
       <c r="J71" t="n">
-        <v>211.6795092945534</v>
+        <v>298</v>
+      </c>
+      <c r="K71" t="n">
+        <v>184.0450638803032</v>
+      </c>
+      <c r="L71" t="n">
+        <v>-3.630966901779175</v>
+      </c>
+      <c r="M71" t="n">
+        <v>294.3690330982208</v>
       </c>
     </row>
     <row r="72">
@@ -3009,19 +3794,30 @@
         <v>19307.24</v>
       </c>
       <c r="F72" t="n">
-        <v>35095</v>
+        <v>15530.26</v>
       </c>
       <c r="G72" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H72" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I72" t="n">
         <v>310</v>
       </c>
-      <c r="H72" t="n">
-        <v>229.9912044684341</v>
-      </c>
-      <c r="I72" t="n">
-        <v>13.17655849456787</v>
-      </c>
       <c r="J72" t="n">
-        <v>243.167762963002</v>
+        <v>310</v>
+      </c>
+      <c r="K72" t="n">
+        <v>213.0960444488196</v>
+      </c>
+      <c r="L72" t="n">
+        <v>0.001408874988555908</v>
+      </c>
+      <c r="M72" t="n">
+        <v>310.0014088749886</v>
       </c>
     </row>
     <row r="73">
@@ -3045,19 +3841,30 @@
         <v>20223.59</v>
       </c>
       <c r="F73" t="n">
-        <v>35095</v>
+        <v>14884.51</v>
       </c>
       <c r="G73" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I73" t="n">
         <v>310</v>
       </c>
-      <c r="H73" t="n">
-        <v>276.6756074573791</v>
-      </c>
-      <c r="I73" t="n">
-        <v>13.17655849456787</v>
-      </c>
       <c r="J73" t="n">
-        <v>289.852165951947</v>
+        <v>310</v>
+      </c>
+      <c r="K73" t="n">
+        <v>239.3852217645793</v>
+      </c>
+      <c r="L73" t="n">
+        <v>0.001408874988555908</v>
+      </c>
+      <c r="M73" t="n">
+        <v>310.0014088749886</v>
       </c>
     </row>
     <row r="74">
@@ -3081,19 +3888,30 @@
         <v>21002.12</v>
       </c>
       <c r="F74" t="n">
-        <v>35095</v>
+        <v>14177.88</v>
       </c>
       <c r="G74" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I74" t="n">
         <v>305</v>
       </c>
-      <c r="H74" t="n">
-        <v>242.027387231861</v>
-      </c>
-      <c r="I74" t="n">
-        <v>13.17655849456787</v>
-      </c>
       <c r="J74" t="n">
-        <v>255.2039457264289</v>
+        <v>305</v>
+      </c>
+      <c r="K74" t="n">
+        <v>239.1450726185516</v>
+      </c>
+      <c r="L74" t="n">
+        <v>-3.630966901779175</v>
+      </c>
+      <c r="M74" t="n">
+        <v>301.3690330982208</v>
       </c>
     </row>
     <row r="75">
@@ -3117,19 +3935,30 @@
         <v>21996.82</v>
       </c>
       <c r="F75" t="n">
-        <v>35095</v>
+        <v>13488.68</v>
       </c>
       <c r="G75" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I75" t="n">
         <v>305</v>
       </c>
-      <c r="H75" t="n">
-        <v>258.3912237021769</v>
-      </c>
-      <c r="I75" t="n">
-        <v>13.17655849456787</v>
-      </c>
       <c r="J75" t="n">
-        <v>271.5677821967448</v>
+        <v>305</v>
+      </c>
+      <c r="K75" t="n">
+        <v>248.2731623617452</v>
+      </c>
+      <c r="L75" t="n">
+        <v>-3.630966901779175</v>
+      </c>
+      <c r="M75" t="n">
+        <v>301.3690330982208</v>
       </c>
     </row>
     <row r="76">
@@ -3153,19 +3982,30 @@
         <v>22809.19</v>
       </c>
       <c r="F76" t="n">
-        <v>35095</v>
+        <v>12831.11</v>
       </c>
       <c r="G76" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I76" t="n">
         <v>330</v>
       </c>
-      <c r="H76" t="n">
-        <v>268.8675142042662</v>
-      </c>
-      <c r="I76" t="n">
-        <v>13.17655849456787</v>
-      </c>
       <c r="J76" t="n">
-        <v>282.044072698834</v>
+        <v>330</v>
+      </c>
+      <c r="K76" t="n">
+        <v>251.8283778868781</v>
+      </c>
+      <c r="L76" t="n">
+        <v>2.622707366943359</v>
+      </c>
+      <c r="M76" t="n">
+        <v>332.6227073669434</v>
       </c>
     </row>
     <row r="77">
@@ -3189,19 +4029,30 @@
         <v>23504.41</v>
       </c>
       <c r="F77" t="n">
-        <v>35095</v>
+        <v>12289.89</v>
       </c>
       <c r="G77" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I77" t="n">
         <v>339</v>
       </c>
-      <c r="H77" t="n">
-        <v>273.7647282256407</v>
-      </c>
-      <c r="I77" t="n">
-        <v>13.17655849456787</v>
-      </c>
       <c r="J77" t="n">
-        <v>286.9412867202086</v>
+        <v>339</v>
+      </c>
+      <c r="K77" t="n">
+        <v>264.4434456541305</v>
+      </c>
+      <c r="L77" t="n">
+        <v>2.622707366943359</v>
+      </c>
+      <c r="M77" t="n">
+        <v>341.6227073669434</v>
       </c>
     </row>
     <row r="78">
@@ -3225,19 +4076,30 @@
         <v>23956.57</v>
       </c>
       <c r="F78" t="n">
-        <v>35095</v>
+        <v>11972.73</v>
       </c>
       <c r="G78" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I78" t="n">
         <v>328</v>
       </c>
-      <c r="H78" t="n">
-        <v>272.3598865510795</v>
-      </c>
-      <c r="I78" t="n">
-        <v>13.17655849456787</v>
-      </c>
       <c r="J78" t="n">
-        <v>285.5364450456474</v>
+        <v>328</v>
+      </c>
+      <c r="K78" t="n">
+        <v>264.1720749048455</v>
+      </c>
+      <c r="L78" t="n">
+        <v>2.622707366943359</v>
+      </c>
+      <c r="M78" t="n">
+        <v>330.6227073669434</v>
       </c>
     </row>
     <row r="79">
@@ -3261,19 +4123,30 @@
         <v>24188.65</v>
       </c>
       <c r="F79" t="n">
-        <v>35095</v>
+        <v>11798.65</v>
       </c>
       <c r="G79" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I79" t="n">
         <v>325</v>
       </c>
-      <c r="H79" t="n">
-        <v>265.3098230351048</v>
-      </c>
-      <c r="I79" t="n">
-        <v>13.17655849456787</v>
-      </c>
       <c r="J79" t="n">
-        <v>278.4863815296727</v>
+        <v>325</v>
+      </c>
+      <c r="K79" t="n">
+        <v>264.0560532600432</v>
+      </c>
+      <c r="L79" t="n">
+        <v>2.622707366943359</v>
+      </c>
+      <c r="M79" t="n">
+        <v>327.6227073669434</v>
       </c>
     </row>
     <row r="80">
@@ -3297,19 +4170,30 @@
         <v>24286.61</v>
       </c>
       <c r="F80" t="n">
-        <v>35095</v>
+        <v>11700.69</v>
       </c>
       <c r="G80" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I80" t="n">
         <v>325</v>
       </c>
-      <c r="H80" t="n">
-        <v>271.2861954404619</v>
-      </c>
-      <c r="I80" t="n">
-        <v>13.17655849456787</v>
-      </c>
       <c r="J80" t="n">
-        <v>284.4627539350298</v>
+        <v>324.9999999999999</v>
+      </c>
+      <c r="K80" t="n">
+        <v>265.5045212794324</v>
+      </c>
+      <c r="L80" t="n">
+        <v>2.622707366943359</v>
+      </c>
+      <c r="M80" t="n">
+        <v>327.6227073669433</v>
       </c>
     </row>
     <row r="81">
@@ -3333,19 +4217,30 @@
         <v>24233.07</v>
       </c>
       <c r="F81" t="n">
-        <v>35095</v>
+        <v>11735.23</v>
       </c>
       <c r="G81" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I81" t="n">
         <v>318</v>
       </c>
-      <c r="H81" t="n">
-        <v>270.4843253974767</v>
-      </c>
-      <c r="I81" t="n">
-        <v>13.17655849456787</v>
-      </c>
       <c r="J81" t="n">
-        <v>283.6608838920445</v>
+        <v>318</v>
+      </c>
+      <c r="K81" t="n">
+        <v>264.7560004290006</v>
+      </c>
+      <c r="L81" t="n">
+        <v>0.001408874988555908</v>
+      </c>
+      <c r="M81" t="n">
+        <v>318.0014088749886</v>
       </c>
     </row>
     <row r="82">
@@ -3369,19 +4264,30 @@
         <v>24216.92</v>
       </c>
       <c r="F82" t="n">
-        <v>35095</v>
+        <v>11674.38</v>
       </c>
       <c r="G82" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H82" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I82" t="n">
         <v>313</v>
       </c>
-      <c r="H82" t="n">
-        <v>269.8281208449547</v>
-      </c>
-      <c r="I82" t="n">
-        <v>7.415987968444824</v>
-      </c>
       <c r="J82" t="n">
-        <v>277.2441088133995</v>
+        <v>313</v>
+      </c>
+      <c r="K82" t="n">
+        <v>264.5267664845981</v>
+      </c>
+      <c r="L82" t="n">
+        <v>21.8750171661377</v>
+      </c>
+      <c r="M82" t="n">
+        <v>334.8750171661377</v>
       </c>
     </row>
     <row r="83">
@@ -3405,19 +4311,30 @@
         <v>23991.79</v>
       </c>
       <c r="F83" t="n">
-        <v>35095</v>
+        <v>11612.51</v>
       </c>
       <c r="G83" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H83" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I83" t="n">
         <v>325</v>
       </c>
-      <c r="H83" t="n">
-        <v>275.3007896207092</v>
-      </c>
-      <c r="I83" t="n">
-        <v>7.415987968444824</v>
-      </c>
       <c r="J83" t="n">
-        <v>282.716777589154</v>
+        <v>325</v>
+      </c>
+      <c r="K83" t="n">
+        <v>264.1374246827615</v>
+      </c>
+      <c r="L83" t="n">
+        <v>23.28093147277832</v>
+      </c>
+      <c r="M83" t="n">
+        <v>348.2809314727783</v>
       </c>
     </row>
     <row r="84">
@@ -3441,19 +4358,30 @@
         <v>23698</v>
       </c>
       <c r="F84" t="n">
-        <v>35095</v>
+        <v>11562.3</v>
       </c>
       <c r="G84" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H84" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I84" t="n">
         <v>318</v>
       </c>
-      <c r="H84" t="n">
-        <v>266.3351306546755</v>
-      </c>
-      <c r="I84" t="n">
-        <v>7.415987968444824</v>
-      </c>
       <c r="J84" t="n">
-        <v>273.7511186231203</v>
+        <v>318</v>
+      </c>
+      <c r="K84" t="n">
+        <v>263.5318165323345</v>
+      </c>
+      <c r="L84" t="n">
+        <v>23.28093147277832</v>
+      </c>
+      <c r="M84" t="n">
+        <v>341.2809314727783</v>
       </c>
     </row>
     <row r="85">
@@ -3477,19 +4405,30 @@
         <v>23332.61</v>
       </c>
       <c r="F85" t="n">
-        <v>35095</v>
+        <v>11563.69</v>
       </c>
       <c r="G85" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H85" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I85" t="n">
         <v>318</v>
       </c>
-      <c r="H85" t="n">
-        <v>263.8748987279326</v>
-      </c>
-      <c r="I85" t="n">
-        <v>7.415987968444824</v>
-      </c>
       <c r="J85" t="n">
-        <v>271.2908866963774</v>
+        <v>318</v>
+      </c>
+      <c r="K85" t="n">
+        <v>262.2504450889737</v>
+      </c>
+      <c r="L85" t="n">
+        <v>23.28093147277832</v>
+      </c>
+      <c r="M85" t="n">
+        <v>341.2809314727783</v>
       </c>
     </row>
     <row r="86">
@@ -3513,19 +4452,30 @@
         <v>22960.57</v>
       </c>
       <c r="F86" t="n">
-        <v>35095</v>
+        <v>11552.73</v>
       </c>
       <c r="G86" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H86" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I86" t="n">
         <v>325</v>
       </c>
-      <c r="H86" t="n">
-        <v>262.6333180197364</v>
-      </c>
-      <c r="I86" t="n">
-        <v>7.415987968444824</v>
-      </c>
       <c r="J86" t="n">
-        <v>270.0493059881812</v>
+        <v>325</v>
+      </c>
+      <c r="K86" t="n">
+        <v>257.8748667315675</v>
+      </c>
+      <c r="L86" t="n">
+        <v>24.38485717773438</v>
+      </c>
+      <c r="M86" t="n">
+        <v>349.3848571777344</v>
       </c>
     </row>
     <row r="87">
@@ -3549,19 +4499,30 @@
         <v>22468.03</v>
       </c>
       <c r="F87" t="n">
-        <v>35095</v>
+        <v>11550.27</v>
       </c>
       <c r="G87" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H87" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I87" t="n">
         <v>300</v>
       </c>
-      <c r="H87" t="n">
-        <v>276.3301368089377</v>
-      </c>
-      <c r="I87" t="n">
-        <v>7.415987968444824</v>
-      </c>
       <c r="J87" t="n">
-        <v>283.7461247773825</v>
+        <v>300</v>
+      </c>
+      <c r="K87" t="n">
+        <v>247.9832908277266</v>
+      </c>
+      <c r="L87" t="n">
+        <v>20.68198013305664</v>
+      </c>
+      <c r="M87" t="n">
+        <v>320.6819801330566</v>
       </c>
     </row>
     <row r="88">
@@ -3585,19 +4546,30 @@
         <v>21896.5</v>
       </c>
       <c r="F88" t="n">
-        <v>35095</v>
+        <v>11548.8</v>
       </c>
       <c r="G88" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H88" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I88" t="n">
         <v>310</v>
       </c>
-      <c r="H88" t="n">
-        <v>257.8474278407156</v>
-      </c>
-      <c r="I88" t="n">
-        <v>7.415987968444824</v>
-      </c>
       <c r="J88" t="n">
-        <v>265.2634158091604</v>
+        <v>310</v>
+      </c>
+      <c r="K88" t="n">
+        <v>248.504095536432</v>
+      </c>
+      <c r="L88" t="n">
+        <v>17.63161849975586</v>
+      </c>
+      <c r="M88" t="n">
+        <v>327.6316184997559</v>
       </c>
     </row>
     <row r="89">
@@ -3621,19 +4593,30 @@
         <v>21374.94</v>
       </c>
       <c r="F89" t="n">
-        <v>35095</v>
+        <v>11555.36</v>
       </c>
       <c r="G89" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H89" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I89" t="n">
         <v>300</v>
       </c>
-      <c r="H89" t="n">
-        <v>253.9053585257404</v>
-      </c>
-      <c r="I89" t="n">
-        <v>7.415987968444824</v>
-      </c>
       <c r="J89" t="n">
-        <v>261.3213464941852</v>
+        <v>300</v>
+      </c>
+      <c r="K89" t="n">
+        <v>249.1512754809166</v>
+      </c>
+      <c r="L89" t="n">
+        <v>13.62749481201172</v>
+      </c>
+      <c r="M89" t="n">
+        <v>313.6274948120117</v>
       </c>
     </row>
     <row r="90">
@@ -3657,19 +4640,30 @@
         <v>20900.98</v>
       </c>
       <c r="F90" t="n">
-        <v>35095</v>
+        <v>11518.32</v>
       </c>
       <c r="G90" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H90" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I90" t="n">
         <v>298</v>
       </c>
-      <c r="H90" t="n">
-        <v>237.1324135419671</v>
-      </c>
-      <c r="I90" t="n">
-        <v>7.415987968444824</v>
-      </c>
       <c r="J90" t="n">
-        <v>244.5484015104119</v>
+        <v>298</v>
+      </c>
+      <c r="K90" t="n">
+        <v>236.5834995245432</v>
+      </c>
+      <c r="L90" t="n">
+        <v>14.91683578491211</v>
+      </c>
+      <c r="M90" t="n">
+        <v>312.9168357849121</v>
       </c>
     </row>
     <row r="91">
@@ -3693,19 +4687,30 @@
         <v>20397.89</v>
       </c>
       <c r="F91" t="n">
-        <v>35095</v>
+        <v>11504.41</v>
       </c>
       <c r="G91" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H91" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I91" t="n">
         <v>295</v>
       </c>
-      <c r="H91" t="n">
-        <v>250.9996960943939</v>
-      </c>
-      <c r="I91" t="n">
-        <v>7.415987968444824</v>
-      </c>
       <c r="J91" t="n">
-        <v>258.4156840628387</v>
+        <v>295</v>
+      </c>
+      <c r="K91" t="n">
+        <v>239.1838475905462</v>
+      </c>
+      <c r="L91" t="n">
+        <v>15.78592872619629</v>
+      </c>
+      <c r="M91" t="n">
+        <v>310.7859287261963</v>
       </c>
     </row>
     <row r="92">
@@ -3729,19 +4734,30 @@
         <v>19911.73</v>
       </c>
       <c r="F92" t="n">
-        <v>35095</v>
+        <v>11492.57</v>
       </c>
       <c r="G92" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H92" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I92" t="n">
         <v>292</v>
       </c>
-      <c r="H92" t="n">
-        <v>236.8127286496897</v>
-      </c>
-      <c r="I92" t="n">
-        <v>7.415987968444824</v>
-      </c>
       <c r="J92" t="n">
-        <v>244.2287166181345</v>
+        <v>292</v>
+      </c>
+      <c r="K92" t="n">
+        <v>235.683692499425</v>
+      </c>
+      <c r="L92" t="n">
+        <v>15.78592872619629</v>
+      </c>
+      <c r="M92" t="n">
+        <v>307.7859287261963</v>
       </c>
     </row>
     <row r="93">
@@ -3765,19 +4781,30 @@
         <v>19478</v>
       </c>
       <c r="F93" t="n">
-        <v>35095</v>
+        <v>11486.3</v>
       </c>
       <c r="G93" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H93" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I93" t="n">
         <v>290</v>
       </c>
-      <c r="H93" t="n">
-        <v>229.6024077029018</v>
-      </c>
-      <c r="I93" t="n">
-        <v>7.415987968444824</v>
-      </c>
       <c r="J93" t="n">
-        <v>237.0183956713466</v>
+        <v>290</v>
+      </c>
+      <c r="K93" t="n">
+        <v>223.5091780752699</v>
+      </c>
+      <c r="L93" t="n">
+        <v>15.78592872619629</v>
+      </c>
+      <c r="M93" t="n">
+        <v>305.7859287261963</v>
       </c>
     </row>
     <row r="94">
@@ -3801,19 +4828,30 @@
         <v>19158.66</v>
       </c>
       <c r="F94" t="n">
-        <v>35095</v>
+        <v>11459.64</v>
       </c>
       <c r="G94" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H94" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I94" t="n">
         <v>275</v>
       </c>
-      <c r="H94" t="n">
-        <v>241.5170041167223</v>
-      </c>
-      <c r="I94" t="n">
-        <v>7.415987968444824</v>
-      </c>
       <c r="J94" t="n">
-        <v>248.9329920851671</v>
+        <v>275</v>
+      </c>
+      <c r="K94" t="n">
+        <v>218.3533350987858</v>
+      </c>
+      <c r="L94" t="n">
+        <v>15.75370979309082</v>
+      </c>
+      <c r="M94" t="n">
+        <v>290.7537097930908</v>
       </c>
     </row>
     <row r="95">
@@ -3837,19 +4875,30 @@
         <v>18973.58</v>
       </c>
       <c r="F95" t="n">
-        <v>35095</v>
+        <v>11429.72</v>
       </c>
       <c r="G95" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H95" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I95" t="n">
         <v>275</v>
       </c>
-      <c r="H95" t="n">
-        <v>233.6456149299366</v>
-      </c>
-      <c r="I95" t="n">
-        <v>7.415987968444824</v>
-      </c>
       <c r="J95" t="n">
-        <v>241.0616028983814</v>
+        <v>275</v>
+      </c>
+      <c r="K95" t="n">
+        <v>218.1009053984058</v>
+      </c>
+      <c r="L95" t="n">
+        <v>15.75370979309082</v>
+      </c>
+      <c r="M95" t="n">
+        <v>290.7537097930908</v>
       </c>
     </row>
     <row r="96">
@@ -3873,19 +4922,30 @@
         <v>18839.18</v>
       </c>
       <c r="F96" t="n">
-        <v>35095</v>
+        <v>11390.12</v>
       </c>
       <c r="G96" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H96" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I96" t="n">
         <v>270</v>
       </c>
-      <c r="H96" t="n">
-        <v>221.5849831213032</v>
-      </c>
-      <c r="I96" t="n">
-        <v>7.415987968444824</v>
-      </c>
       <c r="J96" t="n">
-        <v>229.000971089748</v>
+        <v>270</v>
+      </c>
+      <c r="K96" t="n">
+        <v>219.7745048440841</v>
+      </c>
+      <c r="L96" t="n">
+        <v>15.75370979309082</v>
+      </c>
+      <c r="M96" t="n">
+        <v>285.7537097930908</v>
       </c>
     </row>
     <row r="97">
@@ -3909,19 +4969,30 @@
         <v>19005.17</v>
       </c>
       <c r="F97" t="n">
-        <v>35095</v>
+        <v>11412.13</v>
       </c>
       <c r="G97" t="n">
+        <v>35095</v>
+      </c>
+      <c r="H97" t="inlineStr">
+        <is>
+          <t>weekend</t>
+        </is>
+      </c>
+      <c r="I97" t="n">
         <v>270</v>
       </c>
-      <c r="H97" t="n">
-        <v>237.6219657425447</v>
-      </c>
-      <c r="I97" t="n">
-        <v>7.415987968444824</v>
-      </c>
       <c r="J97" t="n">
-        <v>245.0379537109895</v>
+        <v>270</v>
+      </c>
+      <c r="K97" t="n">
+        <v>217.645133044379</v>
+      </c>
+      <c r="L97" t="n">
+        <v>15.75370979309082</v>
+      </c>
+      <c r="M97" t="n">
+        <v>285.7537097930908</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Add rolling backtest metrics and rerank window search
</commit_message>
<xml_diff>
--- a/output/dayahead_price_prediction.xlsx
+++ b/output/dayahead_price_prediction.xlsx
@@ -542,10 +542,10 @@
         </is>
       </c>
       <c r="N2" t="n">
-        <v>58.03684355882308</v>
+        <v>85.16122714451075</v>
       </c>
       <c r="O2" t="n">
-        <v>315.0368435588231</v>
+        <v>342.1612271445107</v>
       </c>
     </row>
     <row r="3">
@@ -597,10 +597,10 @@
         </is>
       </c>
       <c r="N3" t="n">
-        <v>49.3550680207718</v>
+        <v>70.30135928068864</v>
       </c>
       <c r="O3" t="n">
-        <v>309.3550680207718</v>
+        <v>330.3013592806886</v>
       </c>
     </row>
     <row r="4">
@@ -652,10 +652,10 @@
         </is>
       </c>
       <c r="N4" t="n">
-        <v>45.85003650978848</v>
+        <v>63.45846355472224</v>
       </c>
       <c r="O4" t="n">
-        <v>306.8500365097885</v>
+        <v>324.4584635547222</v>
       </c>
     </row>
     <row r="5">
@@ -707,10 +707,10 @@
         </is>
       </c>
       <c r="N5" t="n">
-        <v>43.11849608782319</v>
+        <v>54.44239074716597</v>
       </c>
       <c r="O5" t="n">
-        <v>302.1184960878232</v>
+        <v>313.442390747166</v>
       </c>
     </row>
     <row r="6">
@@ -762,10 +762,10 @@
         </is>
       </c>
       <c r="N6" t="n">
-        <v>37.53085967594546</v>
+        <v>40.75225592067272</v>
       </c>
       <c r="O6" t="n">
-        <v>297.5308596759455</v>
+        <v>300.7522559206727</v>
       </c>
     </row>
     <row r="7">
@@ -817,10 +817,10 @@
         </is>
       </c>
       <c r="N7" t="n">
-        <v>38.53085967594546</v>
+        <v>41.75225592067272</v>
       </c>
       <c r="O7" t="n">
-        <v>297.5308596759455</v>
+        <v>300.7522559206727</v>
       </c>
     </row>
     <row r="8">
@@ -872,10 +872,10 @@
         </is>
       </c>
       <c r="N8" t="n">
-        <v>37.53085967594546</v>
+        <v>40.75225592067272</v>
       </c>
       <c r="O8" t="n">
-        <v>297.5308596759455</v>
+        <v>300.7522559206727</v>
       </c>
     </row>
     <row r="9">
@@ -927,10 +927,10 @@
         </is>
       </c>
       <c r="N9" t="n">
-        <v>46.85003650978848</v>
+        <v>64.45846355472224</v>
       </c>
       <c r="O9" t="n">
-        <v>306.8500365097885</v>
+        <v>324.4584635547222</v>
       </c>
     </row>
     <row r="10">
@@ -982,10 +982,10 @@
         </is>
       </c>
       <c r="N10" t="n">
-        <v>46.85003650978848</v>
+        <v>64.45846355472224</v>
       </c>
       <c r="O10" t="n">
-        <v>306.8500365097885</v>
+        <v>324.4584635547222</v>
       </c>
     </row>
     <row r="11">
@@ -1037,10 +1037,10 @@
         </is>
       </c>
       <c r="N11" t="n">
-        <v>37.11849608782319</v>
+        <v>48.44239074716597</v>
       </c>
       <c r="O11" t="n">
-        <v>302.1184960878232</v>
+        <v>313.442390747166</v>
       </c>
     </row>
     <row r="12">
@@ -1092,10 +1092,10 @@
         </is>
       </c>
       <c r="N12" t="n">
-        <v>37.53085967594546</v>
+        <v>40.75225592067272</v>
       </c>
       <c r="O12" t="n">
-        <v>297.5308596759455</v>
+        <v>300.7522559206727</v>
       </c>
     </row>
     <row r="13">
@@ -1147,10 +1147,10 @@
         </is>
       </c>
       <c r="N13" t="n">
-        <v>41.53085967594546</v>
+        <v>38.00433491607032</v>
       </c>
       <c r="O13" t="n">
-        <v>297.5308596759455</v>
+        <v>294.0043349160703</v>
       </c>
     </row>
     <row r="14">
@@ -1202,10 +1202,10 @@
         </is>
       </c>
       <c r="N14" t="n">
-        <v>34.01848427930054</v>
+        <v>28.55156640391817</v>
       </c>
       <c r="O14" t="n">
-        <v>294.0184842793005</v>
+        <v>288.5515664039182</v>
       </c>
     </row>
     <row r="15">
@@ -1257,10 +1257,10 @@
         </is>
       </c>
       <c r="N15" t="n">
-        <v>37.80208088444809</v>
+        <v>28.8356568773934</v>
       </c>
       <c r="O15" t="n">
-        <v>287.8020808844481</v>
+        <v>278.8356568773934</v>
       </c>
     </row>
     <row r="16">
@@ -1312,10 +1312,10 @@
         </is>
       </c>
       <c r="N16" t="n">
-        <v>34.93794330294315</v>
+        <v>20.87055589059577</v>
       </c>
       <c r="O16" t="n">
-        <v>284.9379433029432</v>
+        <v>270.8705558905958</v>
       </c>
     </row>
     <row r="17">
@@ -1367,10 +1367,10 @@
         </is>
       </c>
       <c r="N17" t="n">
-        <v>35.3065894369312</v>
+        <v>18.83562851542095</v>
       </c>
       <c r="O17" t="n">
-        <v>285.3065894369312</v>
+        <v>268.835628515421</v>
       </c>
     </row>
     <row r="18">
@@ -1422,10 +1422,10 @@
         </is>
       </c>
       <c r="N18" t="n">
-        <v>37.10600979641515</v>
+        <v>19.83562851542098</v>
       </c>
       <c r="O18" t="n">
-        <v>286.1060097964152</v>
+        <v>268.835628515421</v>
       </c>
     </row>
     <row r="19">
@@ -1477,10 +1477,10 @@
         </is>
       </c>
       <c r="N19" t="n">
-        <v>39.02759766672193</v>
+        <v>19.83562851542098</v>
       </c>
       <c r="O19" t="n">
-        <v>288.0275976667219</v>
+        <v>268.835628515421</v>
       </c>
     </row>
     <row r="20">
@@ -1532,10 +1532,10 @@
         </is>
       </c>
       <c r="N20" t="n">
-        <v>38.02759766672193</v>
+        <v>18.83562851542098</v>
       </c>
       <c r="O20" t="n">
-        <v>288.0275976667219</v>
+        <v>268.835628515421</v>
       </c>
     </row>
     <row r="21">
@@ -1587,10 +1587,10 @@
         </is>
       </c>
       <c r="N21" t="n">
-        <v>43.02759766672193</v>
+        <v>23.83562851542098</v>
       </c>
       <c r="O21" t="n">
-        <v>288.0275976667219</v>
+        <v>268.835628515421</v>
       </c>
     </row>
     <row r="22">
@@ -1642,10 +1642,10 @@
         </is>
       </c>
       <c r="N22" t="n">
-        <v>39.2167972043668</v>
+        <v>20.44542900920902</v>
       </c>
       <c r="O22" t="n">
-        <v>289.2167972043668</v>
+        <v>270.445429009209</v>
       </c>
     </row>
     <row r="23">
@@ -1697,10 +1697,10 @@
         </is>
       </c>
       <c r="N23" t="n">
-        <v>34.2167972043668</v>
+        <v>16.22982353090208</v>
       </c>
       <c r="O23" t="n">
-        <v>289.2167972043668</v>
+        <v>271.2298235309021</v>
       </c>
     </row>
     <row r="24">
@@ -1752,10 +1752,10 @@
         </is>
       </c>
       <c r="N24" t="n">
-        <v>29.2167972043668</v>
+        <v>11.22982353090208</v>
       </c>
       <c r="O24" t="n">
-        <v>289.2167972043668</v>
+        <v>271.2298235309021</v>
       </c>
     </row>
     <row r="25">
@@ -1807,10 +1807,10 @@
         </is>
       </c>
       <c r="N25" t="n">
-        <v>29.2614013456967</v>
+        <v>9.619394150588391</v>
       </c>
       <c r="O25" t="n">
-        <v>285.2614013456967</v>
+        <v>265.6193941505884</v>
       </c>
     </row>
     <row r="26">
@@ -1862,10 +1862,10 @@
         </is>
       </c>
       <c r="N26" t="n">
-        <v>-8.834073107069599</v>
+        <v>-8.357329810800877</v>
       </c>
       <c r="O26" t="n">
-        <v>251.1659268929304</v>
+        <v>251.6426701891991</v>
       </c>
     </row>
     <row r="27">
@@ -1917,10 +1917,10 @@
         </is>
       </c>
       <c r="N27" t="n">
-        <v>-13.86217501216441</v>
+        <v>-24.36300613846802</v>
       </c>
       <c r="O27" t="n">
-        <v>231.1378249878356</v>
+        <v>220.636993861532</v>
       </c>
     </row>
     <row r="28">
@@ -1972,10 +1972,10 @@
         </is>
       </c>
       <c r="N28" t="n">
-        <v>-25.76419593921869</v>
+        <v>-34.4980328417258</v>
       </c>
       <c r="O28" t="n">
-        <v>219.2358040607813</v>
+        <v>210.5019671582742</v>
       </c>
     </row>
     <row r="29">
@@ -2027,10 +2027,10 @@
         </is>
       </c>
       <c r="N29" t="n">
-        <v>-43.23939502534071</v>
+        <v>-52.66250963189808</v>
       </c>
       <c r="O29" t="n">
-        <v>196.7606049746593</v>
+        <v>187.3374903681019</v>
       </c>
     </row>
     <row r="30">
@@ -2082,10 +2082,10 @@
         </is>
       </c>
       <c r="N30" t="n">
-        <v>163.4011969702531</v>
+        <v>173.0832295019736</v>
       </c>
       <c r="O30" t="n">
-        <v>163.4011969702531</v>
+        <v>173.0832295019736</v>
       </c>
     </row>
     <row r="31">
@@ -2137,10 +2137,10 @@
         </is>
       </c>
       <c r="N31" t="n">
-        <v>148.7663816184602</v>
+        <v>168.5289463686265</v>
       </c>
       <c r="O31" t="n">
-        <v>148.7663816184602</v>
+        <v>168.5289463686265</v>
       </c>
     </row>
     <row r="32">
@@ -2192,10 +2192,10 @@
         </is>
       </c>
       <c r="N32" t="n">
-        <v>130.1008037433683</v>
+        <v>150.2221348788136</v>
       </c>
       <c r="O32" t="n">
-        <v>130.1008037433683</v>
+        <v>150.2221348788136</v>
       </c>
     </row>
     <row r="33">
@@ -2247,10 +2247,10 @@
         </is>
       </c>
       <c r="N33" t="n">
-        <v>118.0342258956756</v>
+        <v>114.1436817966828</v>
       </c>
       <c r="O33" t="n">
-        <v>118.0342258956756</v>
+        <v>114.1436817966828</v>
       </c>
     </row>
     <row r="34">
@@ -2302,10 +2302,10 @@
         </is>
       </c>
       <c r="N34" t="n">
-        <v>74.71475600942088</v>
+        <v>75.07115048399876</v>
       </c>
       <c r="O34" t="n">
-        <v>74.71475600942088</v>
+        <v>75.07115048399876</v>
       </c>
     </row>
     <row r="35">
@@ -2357,10 +2357,10 @@
         </is>
       </c>
       <c r="N35" t="n">
-        <v>45.96515496954009</v>
+        <v>43.90153412529514</v>
       </c>
       <c r="O35" t="n">
-        <v>45.96515496954009</v>
+        <v>43.90153412529514</v>
       </c>
     </row>
     <row r="36">
@@ -2412,10 +2412,10 @@
         </is>
       </c>
       <c r="N36" t="n">
-        <v>34.47005023045833</v>
+        <v>34.67128113977921</v>
       </c>
       <c r="O36" t="n">
-        <v>34.47005023045833</v>
+        <v>34.67128113977921</v>
       </c>
     </row>
     <row r="37">
@@ -2467,10 +2467,10 @@
         </is>
       </c>
       <c r="N37" t="n">
-        <v>24.73763033132525</v>
+        <v>30.07256077124964</v>
       </c>
       <c r="O37" t="n">
-        <v>24.73763033132525</v>
+        <v>30.07256077124964</v>
       </c>
     </row>
     <row r="38">
@@ -2522,10 +2522,10 @@
         </is>
       </c>
       <c r="N38" t="n">
-        <v>30.45663215176782</v>
+        <v>28.01902034442318</v>
       </c>
       <c r="O38" t="n">
-        <v>30.45663215176782</v>
+        <v>28.01902034442318</v>
       </c>
     </row>
     <row r="39">
@@ -2577,10 +2577,10 @@
         </is>
       </c>
       <c r="N39" t="n">
-        <v>24.41112678975165</v>
+        <v>27.98634354250433</v>
       </c>
       <c r="O39" t="n">
-        <v>24.41112678975165</v>
+        <v>27.98634354250433</v>
       </c>
     </row>
     <row r="40">
@@ -2632,10 +2632,10 @@
         </is>
       </c>
       <c r="N40" t="n">
-        <v>24.41112678975165</v>
+        <v>27.98634354250433</v>
       </c>
       <c r="O40" t="n">
-        <v>24.41112678975165</v>
+        <v>27.98634354250433</v>
       </c>
     </row>
     <row r="41">
@@ -2687,10 +2687,10 @@
         </is>
       </c>
       <c r="N41" t="n">
-        <v>22.87777858070908</v>
+        <v>27.98634354250433</v>
       </c>
       <c r="O41" t="n">
-        <v>22.87777858070908</v>
+        <v>27.98634354250433</v>
       </c>
     </row>
     <row r="42">
@@ -2742,10 +2742,10 @@
         </is>
       </c>
       <c r="N42" t="n">
-        <v>6.666746065084553</v>
+        <v>4.412166540942394</v>
       </c>
       <c r="O42" t="n">
-        <v>6.666746065084553</v>
+        <v>4.412166540942394</v>
       </c>
     </row>
     <row r="43">
@@ -2797,10 +2797,10 @@
         </is>
       </c>
       <c r="N43" t="n">
-        <v>6.666746065084553</v>
+        <v>4.412166540942394</v>
       </c>
       <c r="O43" t="n">
-        <v>6.666746065084553</v>
+        <v>4.412166540942394</v>
       </c>
     </row>
     <row r="44">
@@ -2852,10 +2852,10 @@
         </is>
       </c>
       <c r="N44" t="n">
-        <v>5.765038096529622</v>
+        <v>4.651209794865522</v>
       </c>
       <c r="O44" t="n">
-        <v>5.765038096529622</v>
+        <v>4.651209794865522</v>
       </c>
     </row>
     <row r="45">
@@ -2907,10 +2907,10 @@
         </is>
       </c>
       <c r="N45" t="n">
-        <v>5.765038096529622</v>
+        <v>4.750475695448202</v>
       </c>
       <c r="O45" t="n">
-        <v>5.765038096529622</v>
+        <v>4.750475695448202</v>
       </c>
     </row>
     <row r="46">
@@ -2962,10 +2962,10 @@
         </is>
       </c>
       <c r="N46" t="n">
-        <v>5.96960180503207</v>
+        <v>4.165870954903582</v>
       </c>
       <c r="O46" t="n">
-        <v>5.96960180503207</v>
+        <v>4.165870954903582</v>
       </c>
     </row>
     <row r="47">
@@ -3017,10 +3017,10 @@
         </is>
       </c>
       <c r="N47" t="n">
-        <v>6.050829541267348</v>
+        <v>4.175482068284865</v>
       </c>
       <c r="O47" t="n">
-        <v>6.050829541267348</v>
+        <v>4.175482068284865</v>
       </c>
     </row>
     <row r="48">
@@ -3072,10 +3072,10 @@
         </is>
       </c>
       <c r="N48" t="n">
-        <v>6.050829541267348</v>
+        <v>4.190356519989933</v>
       </c>
       <c r="O48" t="n">
-        <v>6.050829541267348</v>
+        <v>4.190356519989933</v>
       </c>
     </row>
     <row r="49">
@@ -3127,10 +3127,10 @@
         </is>
       </c>
       <c r="N49" t="n">
-        <v>6.050829541267348</v>
+        <v>4.190356519989933</v>
       </c>
       <c r="O49" t="n">
-        <v>6.050829541267348</v>
+        <v>4.190356519989933</v>
       </c>
     </row>
     <row r="50">
@@ -3182,10 +3182,10 @@
         </is>
       </c>
       <c r="N50" t="n">
-        <v>6.048436622859654</v>
+        <v>4.097002066043302</v>
       </c>
       <c r="O50" t="n">
-        <v>6.048436622859654</v>
+        <v>4.097002066043302</v>
       </c>
     </row>
     <row r="51">
@@ -3237,10 +3237,10 @@
         </is>
       </c>
       <c r="N51" t="n">
-        <v>6.200561416900172</v>
+        <v>4.147616390216498</v>
       </c>
       <c r="O51" t="n">
-        <v>6.200561416900172</v>
+        <v>4.147616390216498</v>
       </c>
     </row>
     <row r="52">
@@ -3292,10 +3292,10 @@
         </is>
       </c>
       <c r="N52" t="n">
-        <v>6.165841417505149</v>
+        <v>4.224165147263662</v>
       </c>
       <c r="O52" t="n">
-        <v>6.165841417505149</v>
+        <v>4.224165147263662</v>
       </c>
     </row>
     <row r="53">
@@ -3347,10 +3347,10 @@
         </is>
       </c>
       <c r="N53" t="n">
-        <v>6.294032130875308</v>
+        <v>4.481527483509637</v>
       </c>
       <c r="O53" t="n">
-        <v>6.294032130875308</v>
+        <v>4.481527483509637</v>
       </c>
     </row>
     <row r="54">
@@ -3402,10 +3402,10 @@
         </is>
       </c>
       <c r="N54" t="n">
-        <v>6.368886705965949</v>
+        <v>4.952917474045989</v>
       </c>
       <c r="O54" t="n">
-        <v>6.368886705965949</v>
+        <v>4.952917474045989</v>
       </c>
     </row>
     <row r="55">
@@ -3457,10 +3457,10 @@
         </is>
       </c>
       <c r="N55" t="n">
-        <v>6.368886705965949</v>
+        <v>4.952917474045989</v>
       </c>
       <c r="O55" t="n">
-        <v>6.368886705965949</v>
+        <v>4.952917474045989</v>
       </c>
     </row>
     <row r="56">
@@ -3512,10 +3512,10 @@
         </is>
       </c>
       <c r="N56" t="n">
-        <v>6.368886705965949</v>
+        <v>4.952917474045989</v>
       </c>
       <c r="O56" t="n">
-        <v>6.368886705965949</v>
+        <v>4.952917474045989</v>
       </c>
     </row>
     <row r="57">
@@ -3567,10 +3567,10 @@
         </is>
       </c>
       <c r="N57" t="n">
-        <v>6.761266303624893</v>
+        <v>5.419943254867903</v>
       </c>
       <c r="O57" t="n">
-        <v>6.761266303624893</v>
+        <v>5.419943254867903</v>
       </c>
     </row>
     <row r="58">
@@ -3622,10 +3622,10 @@
         </is>
       </c>
       <c r="N58" t="n">
-        <v>7.043167546621973</v>
+        <v>6.013489673296974</v>
       </c>
       <c r="O58" t="n">
-        <v>7.043167546621973</v>
+        <v>6.013489673296974</v>
       </c>
     </row>
     <row r="59">
@@ -3677,10 +3677,10 @@
         </is>
       </c>
       <c r="N59" t="n">
-        <v>7.043167546621973</v>
+        <v>5.890296928286318</v>
       </c>
       <c r="O59" t="n">
-        <v>7.043167546621973</v>
+        <v>5.890296928286318</v>
       </c>
     </row>
     <row r="60">
@@ -3732,10 +3732,10 @@
         </is>
       </c>
       <c r="N60" t="n">
-        <v>7.043167546621973</v>
+        <v>5.995532511661011</v>
       </c>
       <c r="O60" t="n">
-        <v>7.043167546621973</v>
+        <v>5.995532511661011</v>
       </c>
     </row>
     <row r="61">
@@ -3787,10 +3787,10 @@
         </is>
       </c>
       <c r="N61" t="n">
-        <v>7.587919765200837</v>
+        <v>5.966892486839356</v>
       </c>
       <c r="O61" t="n">
-        <v>7.587919765200837</v>
+        <v>5.966892486839356</v>
       </c>
     </row>
     <row r="62">
@@ -3842,10 +3842,10 @@
         </is>
       </c>
       <c r="N62" t="n">
-        <v>63.93663052546117</v>
+        <v>62.95260385526851</v>
       </c>
       <c r="O62" t="n">
-        <v>63.93663052546117</v>
+        <v>62.95260385526851</v>
       </c>
     </row>
     <row r="63">
@@ -3897,10 +3897,10 @@
         </is>
       </c>
       <c r="N63" t="n">
-        <v>63.93663052546117</v>
+        <v>62.95260385526851</v>
       </c>
       <c r="O63" t="n">
-        <v>63.93663052546117</v>
+        <v>62.95260385526851</v>
       </c>
     </row>
     <row r="64">
@@ -3952,10 +3952,10 @@
         </is>
       </c>
       <c r="N64" t="n">
-        <v>63.93663052546117</v>
+        <v>62.93131291858415</v>
       </c>
       <c r="O64" t="n">
-        <v>63.93663052546117</v>
+        <v>62.93131291858415</v>
       </c>
     </row>
     <row r="65">
@@ -4007,10 +4007,10 @@
         </is>
       </c>
       <c r="N65" t="n">
-        <v>63.93663052546117</v>
+        <v>62.93131291858415</v>
       </c>
       <c r="O65" t="n">
-        <v>63.93663052546117</v>
+        <v>62.93131291858415</v>
       </c>
     </row>
     <row r="66">
@@ -4062,10 +4062,10 @@
         </is>
       </c>
       <c r="N66" t="n">
-        <v>66.16498022719065</v>
+        <v>64.76294308978092</v>
       </c>
       <c r="O66" t="n">
-        <v>66.16498022719065</v>
+        <v>64.76294308978092</v>
       </c>
     </row>
     <row r="67">
@@ -4117,10 +4117,10 @@
         </is>
       </c>
       <c r="N67" t="n">
-        <v>74.82201542934837</v>
+        <v>79.95813155108786</v>
       </c>
       <c r="O67" t="n">
-        <v>74.82201542934837</v>
+        <v>79.95813155108786</v>
       </c>
     </row>
     <row r="68">
@@ -4172,10 +4172,10 @@
         </is>
       </c>
       <c r="N68" t="n">
-        <v>89.81035447382467</v>
+        <v>86.79904185125963</v>
       </c>
       <c r="O68" t="n">
-        <v>89.81035447382467</v>
+        <v>86.79904185125963</v>
       </c>
     </row>
     <row r="69">
@@ -4227,10 +4227,10 @@
         </is>
       </c>
       <c r="N69" t="n">
-        <v>125.775680966808</v>
+        <v>120.9955429894679</v>
       </c>
       <c r="O69" t="n">
-        <v>125.775680966808</v>
+        <v>120.9955429894679</v>
       </c>
     </row>
     <row r="70">
@@ -4282,10 +4282,10 @@
         </is>
       </c>
       <c r="N70" t="n">
-        <v>164.0131232425192</v>
+        <v>164.9454397842253</v>
       </c>
       <c r="O70" t="n">
-        <v>164.0131232425192</v>
+        <v>164.9454397842253</v>
       </c>
     </row>
     <row r="71">
@@ -4337,10 +4337,10 @@
         </is>
       </c>
       <c r="N71" t="n">
-        <v>202.1950352538448</v>
+        <v>191.7760740783146</v>
       </c>
       <c r="O71" t="n">
-        <v>202.1950352538448</v>
+        <v>191.7760740783146</v>
       </c>
     </row>
     <row r="72">
@@ -4392,10 +4392,10 @@
         </is>
       </c>
       <c r="N72" t="n">
-        <v>-2.250515792486908</v>
+        <v>-14.08590468662192</v>
       </c>
       <c r="O72" t="n">
-        <v>236.3094842075131</v>
+        <v>224.4740953133781</v>
       </c>
     </row>
     <row r="73">
@@ -4447,10 +4447,10 @@
         </is>
       </c>
       <c r="N73" t="n">
-        <v>-4.189436900878491</v>
+        <v>-14.02245240624961</v>
       </c>
       <c r="O73" t="n">
-        <v>255.2505630991215</v>
+        <v>245.4175475937504</v>
       </c>
     </row>
     <row r="74">
@@ -4502,10 +4502,10 @@
         </is>
       </c>
       <c r="N74" t="n">
-        <v>-6.872765968555257</v>
+        <v>-7.072874141435136</v>
       </c>
       <c r="O74" t="n">
-        <v>263.1272340314447</v>
+        <v>262.9271258585649</v>
       </c>
     </row>
     <row r="75">
@@ -4557,10 +4557,10 @@
         </is>
       </c>
       <c r="N75" t="n">
-        <v>28.72738255541907</v>
+        <v>28.58197707450336</v>
       </c>
       <c r="O75" t="n">
-        <v>298.7273825554191</v>
+        <v>298.5819770745034</v>
       </c>
     </row>
     <row r="76">
@@ -4612,10 +4612,10 @@
         </is>
       </c>
       <c r="N76" t="n">
-        <v>19.66380622473355</v>
+        <v>12.81880081816723</v>
       </c>
       <c r="O76" t="n">
-        <v>314.6638062247335</v>
+        <v>307.8188008181672</v>
       </c>
     </row>
     <row r="77">
@@ -4667,10 +4667,10 @@
         </is>
       </c>
       <c r="N77" t="n">
-        <v>6.811662520830851</v>
+        <v>3.448859107872295</v>
       </c>
       <c r="O77" t="n">
-        <v>314.9116625208309</v>
+        <v>311.5488591078723</v>
       </c>
     </row>
     <row r="78">
@@ -4722,10 +4722,10 @@
         </is>
       </c>
       <c r="N78" t="n">
-        <v>-7.121290184093766</v>
+        <v>-9.531435983476626</v>
       </c>
       <c r="O78" t="n">
-        <v>313.8787098159062</v>
+        <v>311.4685640165234</v>
       </c>
     </row>
     <row r="79">
@@ -4777,10 +4777,10 @@
         </is>
       </c>
       <c r="N79" t="n">
-        <v>-2.793355936335729</v>
+        <v>-9.013407242520202</v>
       </c>
       <c r="O79" t="n">
-        <v>322.2066440636643</v>
+        <v>315.9865927574798</v>
       </c>
     </row>
     <row r="80">
@@ -4832,10 +4832,10 @@
         </is>
       </c>
       <c r="N80" t="n">
-        <v>4.644784239686885</v>
+        <v>-1.490781767288013</v>
       </c>
       <c r="O80" t="n">
-        <v>324.6447842396869</v>
+        <v>318.509218232712</v>
       </c>
     </row>
     <row r="81">
@@ -4887,10 +4887,10 @@
         </is>
       </c>
       <c r="N81" t="n">
-        <v>-17.95967911051406</v>
+        <v>-25.11917002786112</v>
       </c>
       <c r="O81" t="n">
-        <v>320.0403208894859</v>
+        <v>312.8808299721389</v>
       </c>
     </row>
     <row r="82">
@@ -4942,10 +4942,10 @@
         </is>
       </c>
       <c r="N82" t="n">
-        <v>-30.87786378073935</v>
+        <v>-26.88985246184359</v>
       </c>
       <c r="O82" t="n">
-        <v>307.1221362192607</v>
+        <v>311.1101475381564</v>
       </c>
     </row>
     <row r="83">
@@ -4997,10 +4997,10 @@
         </is>
       </c>
       <c r="N83" t="n">
-        <v>-28.36748814937312</v>
+        <v>-24.79518436291426</v>
       </c>
       <c r="O83" t="n">
-        <v>301.6325118506269</v>
+        <v>305.2048156370857</v>
       </c>
     </row>
     <row r="84">
@@ -5052,10 +5052,10 @@
         </is>
       </c>
       <c r="N84" t="n">
-        <v>-45.04748814937312</v>
+        <v>-42.34030731883621</v>
       </c>
       <c r="O84" t="n">
-        <v>301.6325118506269</v>
+        <v>304.3396926811638</v>
       </c>
     </row>
     <row r="85">
@@ -5107,10 +5107,10 @@
         </is>
       </c>
       <c r="N85" t="n">
-        <v>-51.17727289895186</v>
+        <v>-47.67440323275741</v>
       </c>
       <c r="O85" t="n">
-        <v>298.8227271010481</v>
+        <v>302.3255967672425</v>
       </c>
     </row>
     <row r="86">
@@ -5162,10 +5162,10 @@
         </is>
       </c>
       <c r="N86" t="n">
-        <v>-70.79245031339866</v>
+        <v>-67.43627140122442</v>
       </c>
       <c r="O86" t="n">
-        <v>297.2075496866013</v>
+        <v>300.5637285987756</v>
       </c>
     </row>
     <row r="87">
@@ -5217,10 +5217,10 @@
         </is>
       </c>
       <c r="N87" t="n">
-        <v>-52.79245031339866</v>
+        <v>-49.43627140122442</v>
       </c>
       <c r="O87" t="n">
-        <v>297.2075496866013</v>
+        <v>300.5637285987756</v>
       </c>
     </row>
     <row r="88">
@@ -5272,10 +5272,10 @@
         </is>
       </c>
       <c r="N88" t="n">
-        <v>-47.79245031339866</v>
+        <v>-45.76767127466957</v>
       </c>
       <c r="O88" t="n">
-        <v>297.2075496866013</v>
+        <v>299.2323287253304</v>
       </c>
     </row>
     <row r="89">
@@ -5327,10 +5327,10 @@
         </is>
       </c>
       <c r="N89" t="n">
-        <v>-56.18981622936178</v>
+        <v>-55.27745947142625</v>
       </c>
       <c r="O89" t="n">
-        <v>293.8101837706382</v>
+        <v>294.7225405285737</v>
       </c>
     </row>
     <row r="90">
@@ -5382,10 +5382,10 @@
         </is>
       </c>
       <c r="N90" t="n">
-        <v>-55.14463723069298</v>
+        <v>-53.75633677999213</v>
       </c>
       <c r="O90" t="n">
-        <v>294.855362769307</v>
+        <v>296.2436632200079</v>
       </c>
     </row>
     <row r="91">
@@ -5437,10 +5437,10 @@
         </is>
       </c>
       <c r="N91" t="n">
-        <v>-83.14463723069298</v>
+        <v>-87.96026634855031</v>
       </c>
       <c r="O91" t="n">
-        <v>294.855362769307</v>
+        <v>290.0397336514497</v>
       </c>
     </row>
     <row r="92">
@@ -5492,10 +5492,10 @@
         </is>
       </c>
       <c r="N92" t="n">
-        <v>-55.14463723069298</v>
+        <v>-62.30269841115938</v>
       </c>
       <c r="O92" t="n">
-        <v>294.855362769307</v>
+        <v>287.6973015888406</v>
       </c>
     </row>
     <row r="93">
@@ -5547,10 +5547,10 @@
         </is>
       </c>
       <c r="N93" t="n">
-        <v>-57.15116761725295</v>
+        <v>-64.80057966987135</v>
       </c>
       <c r="O93" t="n">
-        <v>293.848832382747</v>
+        <v>286.1994203301286</v>
       </c>
     </row>
     <row r="94">
@@ -5602,10 +5602,10 @@
         </is>
       </c>
       <c r="N94" t="n">
-        <v>-56.29877500879979</v>
+        <v>-63.80057966987141</v>
       </c>
       <c r="O94" t="n">
-        <v>293.7012249912002</v>
+        <v>286.1994203301286</v>
       </c>
     </row>
     <row r="95">
@@ -5657,10 +5657,10 @@
         </is>
       </c>
       <c r="N95" t="n">
-        <v>-93.29877500879974</v>
+        <v>-100.8005796698714</v>
       </c>
       <c r="O95" t="n">
-        <v>293.7012249912002</v>
+        <v>286.1994203301286</v>
       </c>
     </row>
     <row r="96">
@@ -5712,10 +5712,10 @@
         </is>
       </c>
       <c r="N96" t="n">
-        <v>-74.29877500879979</v>
+        <v>-81.80057966987141</v>
       </c>
       <c r="O96" t="n">
-        <v>293.7012249912002</v>
+        <v>286.1994203301286</v>
       </c>
     </row>
     <row r="97">
@@ -5767,10 +5767,10 @@
         </is>
       </c>
       <c r="N97" t="n">
-        <v>-51.29877500879979</v>
+        <v>-58.80057966987141</v>
       </c>
       <c r="O97" t="n">
-        <v>293.7012249912002</v>
+        <v>286.1994203301286</v>
       </c>
     </row>
   </sheetData>

</xml_diff>